<commit_message>
Locked in Accruals changes
</commit_message>
<xml_diff>
--- a/data/stx_xlsx/AAK.ST.xlsx
+++ b/data/stx_xlsx/AAK.ST.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="402">
   <si>
     <t>Company Fundamentals - Income Statement</t>
   </si>
@@ -763,6 +763,9 @@
   </si>
   <si>
     <t>Other non-current liabilities</t>
+  </si>
+  <si>
+    <t>Liabilities to banks and credit institutions (Do not use)</t>
   </si>
   <si>
     <t>Pension liabilities</t>
@@ -1347,7 +1350,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1425,6 +1428,9 @@
     </xf>
     <xf borderId="3" fillId="0" fontId="8" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -10425,8 +10431,12 @@
       <c r="S33" s="20">
         <v>86.25</v>
       </c>
-      <c r="T33" s="15"/>
-      <c r="U33" s="15"/>
+      <c r="T33" s="16">
+        <v>140.45</v>
+      </c>
+      <c r="U33" s="16">
+        <v>117.46</v>
+      </c>
       <c r="V33" s="15"/>
     </row>
     <row r="34" ht="15.0" customHeight="1">
@@ -11129,10 +11139,22 @@
       <c r="Q46" s="16">
         <v>2358.29</v>
       </c>
-      <c r="R46" s="15"/>
-      <c r="S46" s="15"/>
-      <c r="T46" s="15"/>
-      <c r="U46" s="15"/>
+      <c r="R46" s="20">
+        <f t="shared" ref="R46:U46" si="1">SUM(R47,R50,R54,R56,R60:R61)</f>
+        <v>2409.53</v>
+      </c>
+      <c r="S46" s="20">
+        <f t="shared" si="1"/>
+        <v>2835.74</v>
+      </c>
+      <c r="T46" s="20">
+        <f t="shared" si="1"/>
+        <v>2492.72</v>
+      </c>
+      <c r="U46" s="20">
+        <f t="shared" si="1"/>
+        <v>2504.85</v>
+      </c>
       <c r="V46" s="15"/>
     </row>
     <row r="47" ht="15.0" customHeight="1">
@@ -13458,8 +13480,8 @@
       <c r="V92" s="15"/>
     </row>
     <row r="93" ht="15.0" customHeight="1">
-      <c r="A93" s="14" t="s">
-        <v>232</v>
+      <c r="A93" s="26" t="s">
+        <v>248</v>
       </c>
       <c r="B93" s="16">
         <v>426.45</v>
@@ -13513,7 +13535,7 @@
     </row>
     <row r="94" ht="15.0" customHeight="1">
       <c r="A94" s="14" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B94" s="20">
         <v>32.8</v>
@@ -13619,7 +13641,7 @@
     </row>
     <row r="96" ht="15.0" customHeight="1">
       <c r="A96" s="14" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B96" s="15"/>
       <c r="C96" s="15"/>
@@ -13649,7 +13671,7 @@
     </row>
     <row r="97" ht="15.0" customHeight="1">
       <c r="A97" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B97" s="16">
         <v>668.11</v>
@@ -13715,7 +13737,7 @@
     </row>
     <row r="98" ht="15.0" customHeight="1">
       <c r="A98" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B98" s="15"/>
       <c r="C98" s="16">
@@ -13845,7 +13867,7 @@
     </row>
     <row r="100" ht="15.0" customHeight="1">
       <c r="A100" s="17" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B100" s="19">
         <v>2067.75</v>
@@ -13911,7 +13933,7 @@
     </row>
     <row r="101" ht="15.0" customHeight="1">
       <c r="A101" s="17" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B101" s="18">
         <v>13836.73</v>
@@ -13977,7 +13999,7 @@
     </row>
     <row r="102" ht="15.0" customHeight="1">
       <c r="A102" s="14" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B102" s="15"/>
       <c r="C102" s="16">
@@ -14041,7 +14063,7 @@
     </row>
     <row r="103" ht="15.0" customHeight="1">
       <c r="A103" s="14" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B103" s="15"/>
       <c r="C103" s="16">
@@ -14105,7 +14127,7 @@
     </row>
     <row r="104" ht="15.0" customHeight="1">
       <c r="A104" s="14" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B104" s="15"/>
       <c r="C104" s="15"/>
@@ -14143,7 +14165,7 @@
     </row>
     <row r="105" ht="15.0" customHeight="1">
       <c r="A105" s="14" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B105" s="15"/>
       <c r="C105" s="20">
@@ -14179,7 +14201,7 @@
     </row>
     <row r="106" ht="15.0" customHeight="1">
       <c r="A106" s="14" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B106" s="15"/>
       <c r="C106" s="15">
@@ -14227,7 +14249,7 @@
     </row>
     <row r="107" ht="15.0" customHeight="1">
       <c r="A107" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B107" s="15"/>
       <c r="C107" s="16">
@@ -14275,7 +14297,7 @@
     </row>
     <row r="108" ht="15.0" customHeight="1">
       <c r="A108" s="14" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B108" s="15"/>
       <c r="C108" s="15"/>
@@ -14303,7 +14325,7 @@
     </row>
     <row r="109" ht="15.0" customHeight="1">
       <c r="A109" s="14" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B109" s="15"/>
       <c r="C109" s="15">
@@ -14367,7 +14389,7 @@
     </row>
     <row r="110" ht="15.0" customHeight="1">
       <c r="A110" s="17" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B110" s="18">
         <v>21756.71</v>
@@ -14499,7 +14521,7 @@
     </row>
     <row r="112" ht="15.0" customHeight="1">
       <c r="A112" s="17" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B112" s="21">
         <v>77.64</v>
@@ -14553,7 +14575,7 @@
     </row>
     <row r="113" ht="15.0" customHeight="1">
       <c r="A113" s="17" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B113" s="18">
         <v>21834.34</v>
@@ -14619,7 +14641,7 @@
     </row>
     <row r="114" ht="15.0" customHeight="1">
       <c r="A114" s="17" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B114" s="18">
         <v>35671.07</v>
@@ -14685,7 +14707,7 @@
     </row>
     <row r="115" ht="15.0" customHeight="1">
       <c r="A115" s="14" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B115" s="16">
         <v>260.45</v>
@@ -14751,7 +14773,7 @@
     </row>
     <row r="116" ht="15.0" customHeight="1">
       <c r="A116" s="14" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B116" s="15">
         <v>0.0</v>
@@ -14817,7 +14839,7 @@
     </row>
     <row r="117" ht="15.0" customHeight="1">
       <c r="A117" s="14" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B117" s="16">
         <v>260.45</v>
@@ -14883,7 +14905,7 @@
     </row>
     <row r="118" ht="15.0" customHeight="1">
       <c r="A118" s="14" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B118" s="15"/>
       <c r="C118" s="15"/>
@@ -14919,7 +14941,7 @@
     </row>
     <row r="119" ht="15.0" customHeight="1">
       <c r="A119" s="14" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B119" s="15"/>
       <c r="C119" s="15"/>
@@ -14953,7 +14975,7 @@
     </row>
     <row r="120" ht="15.0" customHeight="1">
       <c r="A120" s="14" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B120" s="15"/>
       <c r="C120" s="15"/>
@@ -14981,7 +15003,7 @@
     </row>
     <row r="121" ht="15.0" customHeight="1">
       <c r="A121" s="14" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B121" s="15"/>
       <c r="C121" s="15"/>
@@ -15015,7 +15037,7 @@
     </row>
     <row r="122" ht="15.0" customHeight="1">
       <c r="A122" s="14" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B122" s="15"/>
       <c r="C122" s="15"/>
@@ -15043,7 +15065,7 @@
     </row>
     <row r="123" ht="15.0" customHeight="1">
       <c r="A123" s="14" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B123" s="15"/>
       <c r="C123" s="15"/>
@@ -15077,7 +15099,7 @@
     </row>
     <row r="124" ht="15.0" customHeight="1">
       <c r="A124" s="14" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B124" s="15"/>
       <c r="C124" s="16">
@@ -15111,7 +15133,7 @@
     </row>
     <row r="125" ht="15.0" customHeight="1">
       <c r="A125" s="14" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B125" s="15"/>
       <c r="C125" s="16">
@@ -15145,7 +15167,7 @@
     </row>
     <row r="126" ht="15.0" customHeight="1">
       <c r="A126" s="14" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B126" s="15"/>
       <c r="C126" s="15"/>
@@ -15175,7 +15197,7 @@
     </row>
     <row r="127" ht="15.0" customHeight="1">
       <c r="A127" s="14" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B127" s="15"/>
       <c r="C127" s="16">
@@ -15209,7 +15231,7 @@
     </row>
     <row r="128" ht="15.0" customHeight="1">
       <c r="A128" s="14" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B128" s="15"/>
       <c r="C128" s="20">
@@ -15243,7 +15265,7 @@
     </row>
     <row r="129" ht="15.0" customHeight="1">
       <c r="A129" s="14" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B129" s="15"/>
       <c r="C129" s="16">
@@ -15277,7 +15299,7 @@
     </row>
     <row r="130" ht="15.0" customHeight="1">
       <c r="A130" s="14" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B130" s="15"/>
       <c r="C130" s="16">
@@ -15311,7 +15333,7 @@
     </row>
     <row r="131" ht="15.0" customHeight="1">
       <c r="A131" s="14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B131" s="15"/>
       <c r="C131" s="15"/>
@@ -15371,7 +15393,7 @@
     </row>
     <row r="132" ht="15.0" customHeight="1">
       <c r="A132" s="14" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B132" s="15"/>
       <c r="C132" s="15"/>
@@ -15401,7 +15423,7 @@
     </row>
     <row r="133" ht="15.0" customHeight="1">
       <c r="A133" s="14" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B133" s="15"/>
       <c r="C133" s="16">
@@ -15465,7 +15487,7 @@
     </row>
     <row r="134" ht="15.0" customHeight="1">
       <c r="A134" s="14" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B134" s="15"/>
       <c r="C134" s="16">
@@ -15513,7 +15535,7 @@
     </row>
     <row r="135" ht="15.0" customHeight="1">
       <c r="A135" s="14" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B135" s="15"/>
       <c r="C135" s="16">
@@ -15573,7 +15595,7 @@
     </row>
     <row r="136" ht="15.0" customHeight="1">
       <c r="A136" s="14" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B136" s="15"/>
       <c r="C136" s="16">
@@ -15633,7 +15655,7 @@
     </row>
     <row r="137" ht="15.0" customHeight="1">
       <c r="A137" s="14" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B137" s="16">
         <v>260.45</v>
@@ -15699,7 +15721,7 @@
     </row>
     <row r="138" ht="15.0" customHeight="1">
       <c r="A138" s="14" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B138" s="15">
         <v>0.0</v>
@@ -15765,7 +15787,7 @@
     </row>
     <row r="139" ht="15.0" customHeight="1">
       <c r="A139" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B139" s="20">
         <v>1.0</v>
@@ -15831,7 +15853,7 @@
     </row>
     <row r="140" ht="15.0" customHeight="1">
       <c r="A140" s="14" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B140" s="16">
         <v>260.45</v>
@@ -15897,7 +15919,7 @@
     </row>
     <row r="141" ht="15.0" customHeight="1">
       <c r="A141" s="14" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B141" s="15"/>
       <c r="C141" s="15"/>
@@ -15935,7 +15957,7 @@
     </row>
     <row r="142" ht="15.0" customHeight="1">
       <c r="A142" s="14" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B142" s="15"/>
       <c r="C142" s="15"/>
@@ -15987,7 +16009,7 @@
     </row>
     <row r="143" ht="15.0" customHeight="1">
       <c r="A143" s="14" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B143" s="15"/>
       <c r="C143" s="15"/>
@@ -16039,7 +16061,7 @@
     </row>
     <row r="144" ht="15.0" customHeight="1">
       <c r="A144" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B144" s="15"/>
       <c r="C144" s="15"/>
@@ -16091,7 +16113,7 @@
     </row>
     <row r="145" ht="15.0" customHeight="1">
       <c r="A145" s="14" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B145" s="15"/>
       <c r="C145" s="15"/>
@@ -16143,7 +16165,7 @@
     </row>
     <row r="146" ht="15.0" customHeight="1">
       <c r="A146" s="14" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B146" s="15"/>
       <c r="C146" s="15">
@@ -17081,7 +17103,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -17454,67 +17476,67 @@
         <v>43</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="R15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="T15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="V15" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="16" ht="15.0" customHeight="1" outlineLevel="1">
@@ -17587,7 +17609,7 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -17717,7 +17739,7 @@
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="14" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B21" s="15"/>
       <c r="C21" s="16">
@@ -17759,7 +17781,7 @@
     </row>
     <row r="22" ht="15.0" customHeight="1">
       <c r="A22" s="14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="22">
@@ -17791,7 +17813,7 @@
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="14" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
@@ -17827,7 +17849,7 @@
     </row>
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="14" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B24" s="16">
         <v>4089.43</v>
@@ -17877,7 +17899,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="14" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B25" s="16">
         <v>4951.59</v>
@@ -17945,7 +17967,7 @@
     </row>
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="14" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B26" s="15"/>
       <c r="C26" s="16">
@@ -18003,7 +18025,7 @@
     </row>
     <row r="27" ht="15.0" customHeight="1">
       <c r="A27" s="14" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B27" s="22">
         <v>-405.66</v>
@@ -18057,7 +18079,7 @@
     </row>
     <row r="28" ht="15.0" customHeight="1">
       <c r="A28" s="14" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B28" s="15"/>
       <c r="C28" s="15"/>
@@ -18085,7 +18107,7 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="14" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B29" s="15"/>
       <c r="C29" s="15"/>
@@ -18125,7 +18147,7 @@
     </row>
     <row r="30" ht="15.0" customHeight="1">
       <c r="A30" s="14" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
@@ -18163,7 +18185,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="14" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B31" s="15"/>
       <c r="C31" s="15"/>
@@ -18199,7 +18221,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="14" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
@@ -18243,7 +18265,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="14" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B33" s="15"/>
       <c r="C33" s="15"/>
@@ -18285,7 +18307,7 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="14" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B34" s="22">
         <v>-1274.17</v>
@@ -18353,7 +18375,7 @@
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="14" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B35" s="22">
         <v>-116.51</v>
@@ -18383,7 +18405,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="14" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B36" s="22">
         <v>-1323.95</v>
@@ -18451,7 +18473,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="14" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B37" s="22">
         <v>-700.11</v>
@@ -18519,7 +18541,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="14" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B38" s="22">
         <v>-780.6</v>
@@ -18565,7 +18587,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="14" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B39" s="22">
         <v>-371.77</v>
@@ -18619,7 +18641,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="14" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B40" s="22">
         <v>-3176.43</v>
@@ -18667,7 +18689,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="14" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B41" s="15"/>
       <c r="C41" s="15"/>
@@ -18715,7 +18737,7 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="14" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B42" s="15"/>
       <c r="C42" s="15"/>
@@ -18743,7 +18765,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="17" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B43" s="19">
         <v>913.0</v>
@@ -18811,7 +18833,7 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="14" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B44" s="22">
         <v>-1380.09</v>
@@ -18839,7 +18861,7 @@
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="14" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B45" s="15"/>
       <c r="C45" s="23">
@@ -18905,7 +18927,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="14" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B46" s="15"/>
       <c r="C46" s="22">
@@ -18971,7 +18993,7 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="14" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B47" s="15"/>
       <c r="C47" s="15">
@@ -19035,7 +19057,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="14" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B48" s="15">
         <v>0.0</v>
@@ -19065,7 +19087,7 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="14" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B49" s="20">
         <v>8.47</v>
@@ -19133,7 +19155,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="14" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B50" s="15"/>
       <c r="C50" s="15"/>
@@ -19165,7 +19187,7 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="17" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B51" s="25">
         <v>-1371.62</v>
@@ -19233,7 +19255,7 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="14" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B52" s="15"/>
       <c r="C52" s="16">
@@ -19295,7 +19317,7 @@
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="14" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B53" s="15"/>
       <c r="C53" s="22">
@@ -19325,7 +19347,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="14" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B54" s="15"/>
       <c r="C54" s="15"/>
@@ -19373,7 +19395,7 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="14" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B55" s="22">
         <v>-146.16</v>
@@ -19413,7 +19435,7 @@
     </row>
     <row r="56" ht="15.0" customHeight="1">
       <c r="A56" s="14" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B56" s="16">
         <v>185.35</v>
@@ -19457,7 +19479,7 @@
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="14" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B57" s="15"/>
       <c r="C57" s="15"/>
@@ -19495,7 +19517,7 @@
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="14" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B58" s="22">
         <v>-1374.79</v>
@@ -19563,7 +19585,7 @@
     </row>
     <row r="59" ht="15.0" customHeight="1">
       <c r="A59" s="14" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B59" s="16">
         <v>1594.04</v>
@@ -19595,7 +19617,7 @@
     </row>
     <row r="60" ht="15.0" customHeight="1">
       <c r="A60" s="14" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B60" s="15"/>
       <c r="C60" s="15"/>
@@ -19641,7 +19663,7 @@
     </row>
     <row r="61" ht="15.0" customHeight="1">
       <c r="A61" s="14" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B61" s="15"/>
       <c r="C61" s="15"/>
@@ -19671,7 +19693,7 @@
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="17" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B62" s="19">
         <v>258.44</v>
@@ -19739,7 +19761,7 @@
     </row>
     <row r="63" ht="15.0" customHeight="1">
       <c r="A63" s="14" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B63" s="22">
         <v>-200.18</v>
@@ -19793,7 +19815,7 @@
     </row>
     <row r="64" ht="15.0" customHeight="1">
       <c r="A64" s="14" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B64" s="22">
         <v>-165.23</v>
@@ -19861,7 +19883,7 @@
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="14" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B65" s="16">
         <v>2089.61</v>
@@ -19929,7 +19951,7 @@
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="14" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B66" s="16">
         <v>1712.37</v>
@@ -19997,7 +20019,7 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="17" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B67" s="25">
         <v>-365.41</v>
@@ -20065,7 +20087,7 @@
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="14" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B68" s="15"/>
       <c r="C68" s="15"/>
@@ -20105,7 +20127,7 @@
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="14" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B69" s="15"/>
       <c r="C69" s="15"/>
@@ -21094,7 +21116,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -21581,7 +21603,7 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -21670,2541 +21692,2541 @@
       </c>
     </row>
     <row r="20" ht="15.0" customHeight="1">
-      <c r="A20" s="26" t="s">
-        <v>350</v>
-      </c>
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="27"/>
-      <c r="K20" s="27"/>
-      <c r="L20" s="27"/>
-      <c r="M20" s="27"/>
-      <c r="N20" s="27"/>
-      <c r="O20" s="27"/>
-      <c r="P20" s="27"/>
-      <c r="Q20" s="27"/>
-      <c r="R20" s="27"/>
-      <c r="S20" s="27"/>
-      <c r="T20" s="27"/>
-      <c r="U20" s="27"/>
+      <c r="A20" s="27" t="s">
+        <v>351</v>
+      </c>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="28"/>
+      <c r="J20" s="28"/>
+      <c r="K20" s="28"/>
+      <c r="L20" s="28"/>
+      <c r="M20" s="28"/>
+      <c r="N20" s="28"/>
+      <c r="O20" s="28"/>
+      <c r="P20" s="28"/>
+      <c r="Q20" s="28"/>
+      <c r="R20" s="28"/>
+      <c r="S20" s="28"/>
+      <c r="T20" s="28"/>
+      <c r="U20" s="28"/>
     </row>
     <row r="21" ht="15.0" customHeight="1">
-      <c r="A21" s="28" t="s">
-        <v>350</v>
-      </c>
-      <c r="B21" s="29">
+      <c r="A21" s="29" t="s">
+        <v>351</v>
+      </c>
+      <c r="B21" s="30">
         <v>86000.08</v>
       </c>
-      <c r="C21" s="29">
+      <c r="C21" s="30">
         <v>61813.25</v>
       </c>
-      <c r="D21" s="29">
+      <c r="D21" s="30">
         <v>48902.12</v>
       </c>
-      <c r="E21" s="29">
+      <c r="E21" s="30">
         <v>52717.4</v>
       </c>
-      <c r="F21" s="29">
+      <c r="F21" s="30">
         <v>47652.84</v>
       </c>
-      <c r="G21" s="29">
+      <c r="G21" s="30">
         <v>45870.57</v>
       </c>
-      <c r="H21" s="29">
+      <c r="H21" s="30">
         <v>32889.19</v>
       </c>
-      <c r="I21" s="29">
+      <c r="I21" s="30">
         <v>32305.59</v>
       </c>
-      <c r="J21" s="29">
+      <c r="J21" s="30">
         <v>26453.34</v>
       </c>
-      <c r="K21" s="29">
+      <c r="K21" s="30">
         <v>29880.52</v>
       </c>
-      <c r="L21" s="29">
+      <c r="L21" s="30">
         <v>19003.98</v>
       </c>
-      <c r="M21" s="29">
+      <c r="M21" s="30">
         <v>18020.9</v>
       </c>
-      <c r="N21" s="29">
+      <c r="N21" s="30">
         <v>11834.56</v>
       </c>
-      <c r="O21" s="30">
+      <c r="O21" s="31">
         <v>6872.43</v>
       </c>
-      <c r="P21" s="30">
+      <c r="P21" s="31">
         <v>6299.47</v>
       </c>
-      <c r="Q21" s="30">
+      <c r="Q21" s="31">
         <v>5040.79</v>
       </c>
-      <c r="R21" s="30">
+      <c r="R21" s="31">
         <v>4070.6</v>
       </c>
-      <c r="S21" s="30">
+      <c r="S21" s="31">
         <v>4330.23</v>
       </c>
-      <c r="T21" s="30">
+      <c r="T21" s="31">
         <v>8266.78</v>
       </c>
-      <c r="U21" s="30">
+      <c r="U21" s="31">
         <v>6456.55</v>
       </c>
     </row>
     <row r="22" ht="15.0" customHeight="1">
-      <c r="A22" s="28" t="s">
-        <v>351</v>
-      </c>
-      <c r="B22" s="29">
+      <c r="A22" s="29" t="s">
+        <v>352</v>
+      </c>
+      <c r="B22" s="30">
         <v>61016.71</v>
       </c>
-      <c r="C22" s="29">
+      <c r="C22" s="30">
         <v>52757.79</v>
       </c>
-      <c r="D22" s="29">
+      <c r="D22" s="30">
         <v>44111.71</v>
       </c>
-      <c r="E22" s="29">
+      <c r="E22" s="30">
         <v>41826.27</v>
       </c>
-      <c r="F22" s="29">
+      <c r="F22" s="30">
         <v>39353.49</v>
       </c>
-      <c r="G22" s="29">
+      <c r="G22" s="30">
         <v>32134.4</v>
       </c>
-      <c r="H22" s="29">
+      <c r="H22" s="30">
         <v>27765.23</v>
       </c>
-      <c r="I22" s="29">
+      <c r="I22" s="30">
         <v>25552.26</v>
       </c>
-      <c r="J22" s="29">
+      <c r="J22" s="30">
         <v>20714.88</v>
       </c>
-      <c r="K22" s="29">
+      <c r="K22" s="30">
         <v>18679.95</v>
       </c>
-      <c r="L22" s="29">
+      <c r="L22" s="30">
         <v>13026.7</v>
       </c>
-      <c r="M22" s="29">
+      <c r="M22" s="30">
         <v>10245.75</v>
       </c>
-      <c r="N22" s="30">
+      <c r="N22" s="31">
         <v>6816.26</v>
       </c>
-      <c r="O22" s="30">
+      <c r="O22" s="31">
         <v>5403.59</v>
       </c>
-      <c r="P22" s="30">
+      <c r="P22" s="31">
         <v>5604.39</v>
       </c>
-      <c r="Q22" s="30">
+      <c r="Q22" s="31">
         <v>5281.76</v>
       </c>
-      <c r="R22" s="29"/>
-      <c r="S22" s="29"/>
-      <c r="T22" s="29"/>
-      <c r="U22" s="29"/>
+      <c r="R22" s="30"/>
+      <c r="S22" s="30"/>
+      <c r="T22" s="30"/>
+      <c r="U22" s="30"/>
     </row>
     <row r="23" ht="15.0" customHeight="1">
-      <c r="A23" s="26" t="s">
-        <v>352</v>
-      </c>
-      <c r="B23" s="27"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="27"/>
-      <c r="J23" s="27"/>
-      <c r="K23" s="27"/>
-      <c r="L23" s="27"/>
-      <c r="M23" s="27"/>
-      <c r="N23" s="27"/>
-      <c r="O23" s="27"/>
-      <c r="P23" s="27"/>
-      <c r="Q23" s="27"/>
-      <c r="R23" s="27"/>
-      <c r="S23" s="27"/>
-      <c r="T23" s="27"/>
-      <c r="U23" s="27"/>
+      <c r="A23" s="27" t="s">
+        <v>353</v>
+      </c>
+      <c r="B23" s="28"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="28"/>
+      <c r="I23" s="28"/>
+      <c r="J23" s="28"/>
+      <c r="K23" s="28"/>
+      <c r="L23" s="28"/>
+      <c r="M23" s="28"/>
+      <c r="N23" s="28"/>
+      <c r="O23" s="28"/>
+      <c r="P23" s="28"/>
+      <c r="Q23" s="28"/>
+      <c r="R23" s="28"/>
+      <c r="S23" s="28"/>
+      <c r="T23" s="28"/>
+      <c r="U23" s="28"/>
     </row>
     <row r="24" ht="15.0" customHeight="1">
-      <c r="A24" s="28" t="s">
-        <v>352</v>
-      </c>
-      <c r="B24" s="29">
+      <c r="A24" s="29" t="s">
+        <v>353</v>
+      </c>
+      <c r="B24" s="30">
         <v>84218.39</v>
       </c>
-      <c r="C24" s="29">
+      <c r="C24" s="30">
         <v>58743.62</v>
       </c>
-      <c r="D24" s="29">
+      <c r="D24" s="30">
         <v>43451.25</v>
       </c>
-      <c r="E24" s="29">
+      <c r="E24" s="30">
         <v>49186.61</v>
       </c>
-      <c r="F24" s="29">
+      <c r="F24" s="30">
         <v>44272.77</v>
       </c>
-      <c r="G24" s="29">
+      <c r="G24" s="30">
         <v>42348.71</v>
       </c>
-      <c r="H24" s="29">
+      <c r="H24" s="30">
         <v>30381.23</v>
       </c>
-      <c r="I24" s="29">
+      <c r="I24" s="30">
         <v>29726.92</v>
       </c>
-      <c r="J24" s="29">
+      <c r="J24" s="30">
         <v>24041.77</v>
       </c>
-      <c r="K24" s="29">
+      <c r="K24" s="30">
         <v>27771.7</v>
       </c>
-      <c r="L24" s="29">
+      <c r="L24" s="30">
         <v>16694.95</v>
       </c>
-      <c r="M24" s="29">
+      <c r="M24" s="30">
         <v>15967.29</v>
       </c>
-      <c r="N24" s="30">
+      <c r="N24" s="31">
         <v>9662.81</v>
       </c>
-      <c r="O24" s="30">
+      <c r="O24" s="31">
         <v>7079.81</v>
       </c>
-      <c r="P24" s="30">
+      <c r="P24" s="31">
         <v>6689.04</v>
       </c>
-      <c r="Q24" s="30">
+      <c r="Q24" s="31">
         <v>5195.33</v>
       </c>
-      <c r="R24" s="30">
+      <c r="R24" s="31">
         <v>3900.76</v>
       </c>
-      <c r="S24" s="30">
+      <c r="S24" s="31">
         <v>4072.04</v>
       </c>
-      <c r="T24" s="30">
+      <c r="T24" s="31">
         <v>7573.87</v>
       </c>
-      <c r="U24" s="30">
+      <c r="U24" s="31">
         <v>6414.09</v>
       </c>
     </row>
     <row r="25" ht="15.0" customHeight="1">
-      <c r="A25" s="28" t="s">
-        <v>353</v>
-      </c>
-      <c r="B25" s="29">
+      <c r="A25" s="29" t="s">
+        <v>354</v>
+      </c>
+      <c r="B25" s="30">
         <v>57431.94</v>
       </c>
-      <c r="C25" s="29">
+      <c r="C25" s="30">
         <v>48840.07</v>
       </c>
-      <c r="D25" s="29">
+      <c r="D25" s="30">
         <v>40539.04</v>
       </c>
-      <c r="E25" s="29">
+      <c r="E25" s="30">
         <v>38754.56</v>
       </c>
-      <c r="F25" s="29">
+      <c r="F25" s="30">
         <v>36287.09</v>
       </c>
-      <c r="G25" s="29">
+      <c r="G25" s="30">
         <v>29610.02</v>
       </c>
-      <c r="H25" s="29">
+      <c r="H25" s="30">
         <v>25400.91</v>
       </c>
-      <c r="I25" s="29">
+      <c r="I25" s="30">
         <v>23206.14</v>
       </c>
-      <c r="J25" s="29">
+      <c r="J25" s="30">
         <v>18499.04</v>
       </c>
-      <c r="K25" s="29">
+      <c r="K25" s="30">
         <v>16816.85</v>
       </c>
-      <c r="L25" s="29">
+      <c r="L25" s="30">
         <v>11792.72</v>
       </c>
-      <c r="M25" s="30">
+      <c r="M25" s="31">
         <v>9522.51</v>
       </c>
-      <c r="N25" s="30">
+      <c r="N25" s="31">
         <v>6499.7</v>
       </c>
-      <c r="O25" s="30">
+      <c r="O25" s="31">
         <v>5469.71</v>
       </c>
-      <c r="P25" s="30">
+      <c r="P25" s="31">
         <v>5496.97</v>
       </c>
-      <c r="Q25" s="30">
+      <c r="Q25" s="31">
         <v>5100.85</v>
       </c>
-      <c r="R25" s="29"/>
-      <c r="S25" s="29"/>
-      <c r="T25" s="29"/>
-      <c r="U25" s="29"/>
+      <c r="R25" s="30"/>
+      <c r="S25" s="30"/>
+      <c r="T25" s="30"/>
+      <c r="U25" s="30"/>
     </row>
     <row r="26" ht="15.0" customHeight="1">
-      <c r="A26" s="26" t="s">
-        <v>354</v>
-      </c>
-      <c r="B26" s="27"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="27"/>
-      <c r="F26" s="27"/>
-      <c r="G26" s="27"/>
-      <c r="H26" s="27"/>
-      <c r="I26" s="27"/>
-      <c r="J26" s="27"/>
-      <c r="K26" s="27"/>
-      <c r="L26" s="27"/>
-      <c r="M26" s="27"/>
-      <c r="N26" s="27"/>
-      <c r="O26" s="27"/>
-      <c r="P26" s="27"/>
-      <c r="Q26" s="27"/>
-      <c r="R26" s="27"/>
-      <c r="S26" s="27"/>
-      <c r="T26" s="27"/>
-      <c r="U26" s="27"/>
+      <c r="A26" s="27" t="s">
+        <v>355</v>
+      </c>
+      <c r="B26" s="28"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="28"/>
+      <c r="E26" s="28"/>
+      <c r="F26" s="28"/>
+      <c r="G26" s="28"/>
+      <c r="H26" s="28"/>
+      <c r="I26" s="28"/>
+      <c r="J26" s="28"/>
+      <c r="K26" s="28"/>
+      <c r="L26" s="28"/>
+      <c r="M26" s="28"/>
+      <c r="N26" s="28"/>
+      <c r="O26" s="28"/>
+      <c r="P26" s="28"/>
+      <c r="Q26" s="28"/>
+      <c r="R26" s="28"/>
+      <c r="S26" s="28"/>
+      <c r="T26" s="28"/>
+      <c r="U26" s="28"/>
     </row>
     <row r="27" ht="15.0" customHeight="1">
-      <c r="A27" s="28" t="s">
-        <v>355</v>
-      </c>
-      <c r="B27" s="30">
+      <c r="A27" s="29" t="s">
+        <v>356</v>
+      </c>
+      <c r="B27" s="31">
         <v>324.47</v>
       </c>
-      <c r="C27" s="30">
+      <c r="C27" s="31">
         <v>226.32</v>
       </c>
-      <c r="D27" s="30">
+      <c r="D27" s="31">
         <v>167.4</v>
       </c>
-      <c r="E27" s="30">
+      <c r="E27" s="31">
         <v>190.28</v>
       </c>
-      <c r="F27" s="30">
+      <c r="F27" s="31">
         <v>173.34</v>
       </c>
-      <c r="G27" s="30">
+      <c r="G27" s="31">
         <v>166.9</v>
       </c>
-      <c r="H27" s="30">
+      <c r="H27" s="31">
         <v>119.74</v>
       </c>
-      <c r="I27" s="30">
+      <c r="I27" s="31">
         <v>117.16</v>
       </c>
-      <c r="J27" s="31">
+      <c r="J27" s="32">
         <v>94.75</v>
       </c>
-      <c r="K27" s="30">
+      <c r="K27" s="31">
         <v>109.45</v>
       </c>
-      <c r="L27" s="31">
+      <c r="L27" s="32">
         <v>66.7</v>
       </c>
-      <c r="M27" s="31">
+      <c r="M27" s="32">
         <v>64.72</v>
       </c>
-      <c r="N27" s="31">
+      <c r="N27" s="32">
         <v>39.38</v>
       </c>
-      <c r="O27" s="31">
+      <c r="O27" s="32">
         <v>28.85</v>
       </c>
-      <c r="P27" s="31">
+      <c r="P27" s="32">
         <v>27.26</v>
       </c>
-      <c r="Q27" s="31">
+      <c r="Q27" s="32">
         <v>21.17</v>
       </c>
-      <c r="R27" s="31">
+      <c r="R27" s="32">
         <v>15.71</v>
       </c>
-      <c r="S27" s="31">
+      <c r="S27" s="32">
         <v>16.4</v>
       </c>
-      <c r="T27" s="31">
+      <c r="T27" s="32">
         <v>30.5</v>
       </c>
-      <c r="U27" s="31">
+      <c r="U27" s="32">
         <v>26.18</v>
       </c>
     </row>
     <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="28" t="s">
-        <v>356</v>
-      </c>
-      <c r="B28" s="30">
+      <c r="A28" s="29" t="s">
+        <v>357</v>
+      </c>
+      <c r="B28" s="31">
         <v>221.98</v>
       </c>
-      <c r="C28" s="30">
+      <c r="C28" s="31">
         <v>189.66</v>
       </c>
-      <c r="D28" s="30">
+      <c r="D28" s="31">
         <v>158.1</v>
       </c>
-      <c r="E28" s="30">
+      <c r="E28" s="31">
         <v>151.81</v>
       </c>
-      <c r="F28" s="30">
+      <c r="F28" s="31">
         <v>142.78</v>
       </c>
-      <c r="G28" s="30">
+      <c r="G28" s="31">
         <v>116.7</v>
       </c>
-      <c r="H28" s="30">
+      <c r="H28" s="31">
         <v>100.29</v>
       </c>
-      <c r="I28" s="31">
+      <c r="I28" s="32">
         <v>92.03</v>
       </c>
-      <c r="J28" s="31">
+      <c r="J28" s="32">
         <v>73.73</v>
       </c>
-      <c r="K28" s="31">
+      <c r="K28" s="32">
         <v>67.42</v>
       </c>
-      <c r="L28" s="31">
+      <c r="L28" s="32">
         <v>47.72</v>
       </c>
-      <c r="M28" s="31">
+      <c r="M28" s="32">
         <v>38.73</v>
       </c>
-      <c r="N28" s="31">
+      <c r="N28" s="32">
         <v>26.45</v>
       </c>
-      <c r="O28" s="31">
+      <c r="O28" s="32">
         <v>22.21</v>
       </c>
-      <c r="P28" s="31">
+      <c r="P28" s="32">
         <v>22.26</v>
       </c>
-      <c r="Q28" s="31">
+      <c r="Q28" s="32">
         <v>20.66</v>
       </c>
-      <c r="R28" s="29"/>
-      <c r="S28" s="29"/>
-      <c r="T28" s="29"/>
-      <c r="U28" s="29"/>
+      <c r="R28" s="30"/>
+      <c r="S28" s="30"/>
+      <c r="T28" s="30"/>
+      <c r="U28" s="30"/>
     </row>
     <row r="29" ht="15.0" customHeight="1">
-      <c r="A29" s="26" t="s">
-        <v>357</v>
-      </c>
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="27"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="27"/>
-      <c r="I29" s="27"/>
-      <c r="J29" s="27"/>
-      <c r="K29" s="27"/>
-      <c r="L29" s="27"/>
-      <c r="M29" s="27"/>
-      <c r="N29" s="27"/>
-      <c r="O29" s="27"/>
-      <c r="P29" s="27"/>
-      <c r="Q29" s="27"/>
-      <c r="R29" s="27"/>
-      <c r="S29" s="27"/>
-      <c r="T29" s="27"/>
-      <c r="U29" s="27"/>
+      <c r="A29" s="27" t="s">
+        <v>358</v>
+      </c>
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="28"/>
+      <c r="I29" s="28"/>
+      <c r="J29" s="28"/>
+      <c r="K29" s="28"/>
+      <c r="L29" s="28"/>
+      <c r="M29" s="28"/>
+      <c r="N29" s="28"/>
+      <c r="O29" s="28"/>
+      <c r="P29" s="28"/>
+      <c r="Q29" s="28"/>
+      <c r="R29" s="28"/>
+      <c r="S29" s="28"/>
+      <c r="T29" s="28"/>
+      <c r="U29" s="28"/>
     </row>
     <row r="30" ht="15.0" customHeight="1">
-      <c r="A30" s="28" t="s">
-        <v>358</v>
-      </c>
-      <c r="B30" s="32">
+      <c r="A30" s="29" t="s">
+        <v>359</v>
+      </c>
+      <c r="B30" s="33">
         <v>1.35</v>
       </c>
-      <c r="C30" s="32">
+      <c r="C30" s="33">
         <v>6.97</v>
       </c>
-      <c r="D30" s="33">
+      <c r="D30" s="34">
         <v>-2.82</v>
       </c>
-      <c r="E30" s="33">
+      <c r="E30" s="34">
         <v>-0.22</v>
       </c>
-      <c r="F30" s="32">
+      <c r="F30" s="33">
         <v>3.04</v>
       </c>
-      <c r="G30" s="32">
+      <c r="G30" s="33">
         <v>1.68</v>
       </c>
-      <c r="H30" s="32">
+      <c r="H30" s="33">
         <v>1.17</v>
       </c>
-      <c r="I30" s="32">
+      <c r="I30" s="33">
         <v>0.95</v>
       </c>
-      <c r="J30" s="32">
+      <c r="J30" s="33">
         <v>0.93</v>
       </c>
-      <c r="K30" s="32">
+      <c r="K30" s="33">
         <v>2.81</v>
       </c>
-      <c r="L30" s="32">
+      <c r="L30" s="33">
         <v>0.54</v>
       </c>
-      <c r="M30" s="32">
+      <c r="M30" s="33">
         <v>4.35</v>
       </c>
-      <c r="N30" s="32">
+      <c r="N30" s="33">
         <v>10.01</v>
       </c>
-      <c r="O30" s="33">
+      <c r="O30" s="34">
         <v>-8.26</v>
       </c>
-      <c r="P30" s="32">
+      <c r="P30" s="33">
         <v>5.47</v>
       </c>
-      <c r="Q30" s="32">
+      <c r="Q30" s="33">
         <v>30.35</v>
       </c>
-      <c r="R30" s="33">
+      <c r="R30" s="34">
         <v>-8.63</v>
       </c>
-      <c r="S30" s="33">
+      <c r="S30" s="34">
         <v>-20.46</v>
       </c>
-      <c r="T30" s="33">
+      <c r="T30" s="34">
         <v>-3.5</v>
       </c>
-      <c r="U30" s="32"/>
+      <c r="U30" s="33"/>
     </row>
     <row r="31" ht="15.0" customHeight="1">
-      <c r="A31" s="28" t="s">
-        <v>359</v>
-      </c>
-      <c r="B31" s="32">
+      <c r="A31" s="29" t="s">
+        <v>360</v>
+      </c>
+      <c r="B31" s="33">
         <v>1.81</v>
       </c>
-      <c r="C31" s="32">
+      <c r="C31" s="33">
         <v>1.94</v>
       </c>
-      <c r="D31" s="32">
+      <c r="D31" s="33">
         <v>0.48</v>
       </c>
-      <c r="E31" s="32">
+      <c r="E31" s="33">
         <v>1.3</v>
       </c>
-      <c r="F31" s="32">
+      <c r="F31" s="33">
         <v>1.68</v>
       </c>
-      <c r="G31" s="32">
+      <c r="G31" s="33">
         <v>1.51</v>
       </c>
-      <c r="H31" s="32">
+      <c r="H31" s="33">
         <v>1.32</v>
       </c>
-      <c r="I31" s="32">
+      <c r="I31" s="33">
         <v>1.81</v>
       </c>
-      <c r="J31" s="32">
+      <c r="J31" s="33">
         <v>3.04</v>
       </c>
-      <c r="K31" s="32">
+      <c r="K31" s="33">
         <v>2.53</v>
       </c>
-      <c r="L31" s="32">
+      <c r="L31" s="33">
         <v>2.79</v>
       </c>
-      <c r="M31" s="32">
+      <c r="M31" s="33">
         <v>7.06</v>
       </c>
-      <c r="N31" s="32">
+      <c r="N31" s="33">
         <v>6.47</v>
       </c>
-      <c r="O31" s="32">
+      <c r="O31" s="33">
         <v>1.1</v>
       </c>
-      <c r="P31" s="32">
+      <c r="P31" s="33">
         <v>2.32</v>
       </c>
-      <c r="Q31" s="32"/>
-      <c r="R31" s="32"/>
-      <c r="S31" s="32"/>
-      <c r="T31" s="32"/>
-      <c r="U31" s="32"/>
+      <c r="Q31" s="33"/>
+      <c r="R31" s="33"/>
+      <c r="S31" s="33"/>
+      <c r="T31" s="33"/>
+      <c r="U31" s="33"/>
     </row>
     <row r="32" ht="15.0" customHeight="1">
-      <c r="A32" s="26" t="s">
-        <v>360</v>
-      </c>
-      <c r="B32" s="27"/>
-      <c r="C32" s="27"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="27"/>
-      <c r="H32" s="27"/>
-      <c r="I32" s="27"/>
-      <c r="J32" s="27"/>
-      <c r="K32" s="27"/>
-      <c r="L32" s="27"/>
-      <c r="M32" s="27"/>
-      <c r="N32" s="27"/>
-      <c r="O32" s="27"/>
-      <c r="P32" s="27"/>
-      <c r="Q32" s="27"/>
-      <c r="R32" s="27"/>
-      <c r="S32" s="27"/>
-      <c r="T32" s="27"/>
-      <c r="U32" s="27"/>
+      <c r="A32" s="27" t="s">
+        <v>361</v>
+      </c>
+      <c r="B32" s="28"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="28"/>
+      <c r="I32" s="28"/>
+      <c r="J32" s="28"/>
+      <c r="K32" s="28"/>
+      <c r="L32" s="28"/>
+      <c r="M32" s="28"/>
+      <c r="N32" s="28"/>
+      <c r="O32" s="28"/>
+      <c r="P32" s="28"/>
+      <c r="Q32" s="28"/>
+      <c r="R32" s="28"/>
+      <c r="S32" s="28"/>
+      <c r="T32" s="28"/>
+      <c r="U32" s="28"/>
     </row>
     <row r="33" ht="15.0" customHeight="1">
-      <c r="A33" s="28" t="s">
-        <v>361</v>
-      </c>
-      <c r="B33" s="32">
+      <c r="A33" s="29" t="s">
+        <v>362</v>
+      </c>
+      <c r="B33" s="33">
         <v>0.82</v>
       </c>
-      <c r="C33" s="32">
+      <c r="C33" s="33">
         <v>0.86</v>
       </c>
-      <c r="D33" s="32">
+      <c r="D33" s="33">
         <v>0.98</v>
       </c>
-      <c r="E33" s="32">
+      <c r="E33" s="33">
         <v>0.82</v>
       </c>
-      <c r="F33" s="32">
+      <c r="F33" s="33">
         <v>0.89</v>
       </c>
-      <c r="G33" s="32">
+      <c r="G33" s="33">
         <v>0.73</v>
       </c>
-      <c r="H33" s="32">
+      <c r="H33" s="33">
         <v>0.93</v>
       </c>
-      <c r="I33" s="32">
+      <c r="I33" s="33">
         <v>0.87</v>
       </c>
-      <c r="J33" s="32">
+      <c r="J33" s="33">
         <v>0.9</v>
       </c>
-      <c r="K33" s="32">
+      <c r="K33" s="33">
         <v>0.75</v>
       </c>
-      <c r="L33" s="32">
+      <c r="L33" s="33">
         <v>1.01</v>
       </c>
-      <c r="M33" s="32">
+      <c r="M33" s="33">
         <v>0.89</v>
       </c>
-      <c r="N33" s="32">
+      <c r="N33" s="33">
         <v>1.2</v>
       </c>
-      <c r="O33" s="32">
+      <c r="O33" s="33">
         <v>1.58</v>
       </c>
-      <c r="P33" s="32">
+      <c r="P33" s="33">
         <v>1.58</v>
       </c>
-      <c r="Q33" s="32">
+      <c r="Q33" s="33">
         <v>1.78</v>
       </c>
-      <c r="R33" s="32">
+      <c r="R33" s="33">
         <v>2.64</v>
       </c>
-      <c r="S33" s="32">
+      <c r="S33" s="33">
         <v>2.39</v>
       </c>
-      <c r="T33" s="32">
+      <c r="T33" s="33">
         <v>10.1</v>
       </c>
-      <c r="U33" s="32"/>
+      <c r="U33" s="33"/>
     </row>
     <row r="34" ht="15.0" customHeight="1">
-      <c r="A34" s="28" t="s">
-        <v>362</v>
-      </c>
-      <c r="B34" s="32">
+      <c r="A34" s="29" t="s">
+        <v>363</v>
+      </c>
+      <c r="B34" s="33">
         <v>0.87</v>
       </c>
-      <c r="C34" s="32">
+      <c r="C34" s="33">
         <v>0.85</v>
       </c>
-      <c r="D34" s="32">
+      <c r="D34" s="33">
         <v>0.86</v>
       </c>
-      <c r="E34" s="32">
+      <c r="E34" s="33">
         <v>0.84</v>
       </c>
-      <c r="F34" s="32">
+      <c r="F34" s="33">
         <v>0.85</v>
       </c>
-      <c r="G34" s="32">
+      <c r="G34" s="33">
         <v>0.83</v>
       </c>
-      <c r="H34" s="32">
+      <c r="H34" s="33">
         <v>0.89</v>
       </c>
-      <c r="I34" s="32">
+      <c r="I34" s="33">
         <v>0.88</v>
       </c>
-      <c r="J34" s="32">
+      <c r="J34" s="33">
         <v>0.92</v>
       </c>
-      <c r="K34" s="32">
+      <c r="K34" s="33">
         <v>0.99</v>
       </c>
-      <c r="L34" s="32">
+      <c r="L34" s="33">
         <v>1.16</v>
       </c>
-      <c r="M34" s="32">
+      <c r="M34" s="33">
         <v>1.29</v>
       </c>
-      <c r="N34" s="32">
+      <c r="N34" s="33">
         <v>1.62</v>
       </c>
-      <c r="O34" s="32">
+      <c r="O34" s="33">
         <v>1.89</v>
       </c>
-      <c r="P34" s="32">
+      <c r="P34" s="33">
         <v>4.12</v>
       </c>
-      <c r="Q34" s="32"/>
-      <c r="R34" s="32"/>
-      <c r="S34" s="32"/>
-      <c r="T34" s="32"/>
-      <c r="U34" s="32"/>
+      <c r="Q34" s="33"/>
+      <c r="R34" s="33"/>
+      <c r="S34" s="33"/>
+      <c r="T34" s="33"/>
+      <c r="U34" s="33"/>
     </row>
     <row r="35" ht="15.0" customHeight="1">
-      <c r="A35" s="28" t="s">
-        <v>363</v>
-      </c>
-      <c r="B35" s="32">
+      <c r="A35" s="29" t="s">
+        <v>364</v>
+      </c>
+      <c r="B35" s="33">
         <v>1.17</v>
       </c>
-      <c r="C35" s="32">
+      <c r="C35" s="33">
         <v>1.22</v>
       </c>
-      <c r="D35" s="32">
+      <c r="D35" s="33">
         <v>1.41</v>
       </c>
-      <c r="E35" s="32">
+      <c r="E35" s="33">
         <v>1.18</v>
       </c>
-      <c r="F35" s="32">
+      <c r="F35" s="33">
         <v>1.27</v>
       </c>
-      <c r="G35" s="32">
+      <c r="G35" s="33">
         <v>1.04</v>
       </c>
-      <c r="H35" s="32">
+      <c r="H35" s="33">
         <v>1.32</v>
       </c>
-      <c r="I35" s="32">
+      <c r="I35" s="33">
         <v>1.25</v>
       </c>
-      <c r="J35" s="32">
+      <c r="J35" s="33">
         <v>1.29</v>
       </c>
-      <c r="K35" s="32">
+      <c r="K35" s="33">
         <v>1.08</v>
       </c>
-      <c r="L35" s="32">
+      <c r="L35" s="33">
         <v>1.44</v>
       </c>
-      <c r="M35" s="32">
+      <c r="M35" s="33">
         <v>1.27</v>
       </c>
-      <c r="N35" s="32">
+      <c r="N35" s="33">
         <v>1.72</v>
       </c>
-      <c r="O35" s="32">
+      <c r="O35" s="33">
         <v>2.26</v>
       </c>
-      <c r="P35" s="32">
+      <c r="P35" s="33">
         <v>2.25</v>
       </c>
-      <c r="Q35" s="32">
+      <c r="Q35" s="33">
         <v>2.55</v>
       </c>
-      <c r="R35" s="32">
+      <c r="R35" s="33">
         <v>3.77</v>
       </c>
-      <c r="S35" s="32">
+      <c r="S35" s="33">
         <v>3.42</v>
       </c>
-      <c r="T35" s="32">
+      <c r="T35" s="33">
         <v>14.43</v>
       </c>
-      <c r="U35" s="32"/>
+      <c r="U35" s="33"/>
     </row>
     <row r="36" ht="15.0" customHeight="1">
-      <c r="A36" s="28" t="s">
-        <v>364</v>
-      </c>
-      <c r="B36" s="32">
+      <c r="A36" s="29" t="s">
+        <v>365</v>
+      </c>
+      <c r="B36" s="33">
         <v>1.24</v>
       </c>
-      <c r="C36" s="32">
+      <c r="C36" s="33">
         <v>1.22</v>
       </c>
-      <c r="D36" s="32">
+      <c r="D36" s="33">
         <v>1.24</v>
       </c>
-      <c r="E36" s="32">
+      <c r="E36" s="33">
         <v>1.2</v>
       </c>
-      <c r="F36" s="32">
+      <c r="F36" s="33">
         <v>1.22</v>
       </c>
-      <c r="G36" s="32">
+      <c r="G36" s="33">
         <v>1.18</v>
       </c>
-      <c r="H36" s="32">
+      <c r="H36" s="33">
         <v>1.26</v>
       </c>
-      <c r="I36" s="32">
+      <c r="I36" s="33">
         <v>1.25</v>
       </c>
-      <c r="J36" s="32">
+      <c r="J36" s="33">
         <v>1.31</v>
       </c>
-      <c r="K36" s="32">
+      <c r="K36" s="33">
         <v>1.41</v>
       </c>
-      <c r="L36" s="32">
+      <c r="L36" s="33">
         <v>1.66</v>
       </c>
-      <c r="M36" s="32">
+      <c r="M36" s="33">
         <v>1.85</v>
       </c>
-      <c r="N36" s="32">
+      <c r="N36" s="33">
         <v>2.32</v>
       </c>
-      <c r="O36" s="32">
+      <c r="O36" s="33">
         <v>2.7</v>
       </c>
-      <c r="P36" s="32">
+      <c r="P36" s="33">
         <v>5.88</v>
       </c>
-      <c r="Q36" s="32"/>
-      <c r="R36" s="32"/>
-      <c r="S36" s="32"/>
-      <c r="T36" s="32"/>
-      <c r="U36" s="32"/>
+      <c r="Q36" s="33"/>
+      <c r="R36" s="33"/>
+      <c r="S36" s="33"/>
+      <c r="T36" s="33"/>
+      <c r="U36" s="33"/>
     </row>
     <row r="37" ht="15.0" customHeight="1">
-      <c r="A37" s="26" t="s">
-        <v>365</v>
-      </c>
-      <c r="B37" s="27"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="27"/>
-      <c r="G37" s="27"/>
-      <c r="H37" s="27"/>
-      <c r="I37" s="27"/>
-      <c r="J37" s="27"/>
-      <c r="K37" s="27"/>
-      <c r="L37" s="27"/>
-      <c r="M37" s="27"/>
-      <c r="N37" s="27"/>
-      <c r="O37" s="27"/>
-      <c r="P37" s="27"/>
-      <c r="Q37" s="27"/>
-      <c r="R37" s="27"/>
-      <c r="S37" s="27"/>
-      <c r="T37" s="27"/>
-      <c r="U37" s="27"/>
+      <c r="A37" s="27" t="s">
+        <v>366</v>
+      </c>
+      <c r="B37" s="28"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="28"/>
+      <c r="G37" s="28"/>
+      <c r="H37" s="28"/>
+      <c r="I37" s="28"/>
+      <c r="J37" s="28"/>
+      <c r="K37" s="28"/>
+      <c r="L37" s="28"/>
+      <c r="M37" s="28"/>
+      <c r="N37" s="28"/>
+      <c r="O37" s="28"/>
+      <c r="P37" s="28"/>
+      <c r="Q37" s="28"/>
+      <c r="R37" s="28"/>
+      <c r="S37" s="28"/>
+      <c r="T37" s="28"/>
+      <c r="U37" s="28"/>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="28" t="s">
-        <v>366</v>
-      </c>
-      <c r="B38" s="31">
+      <c r="A38" s="29" t="s">
+        <v>367</v>
+      </c>
+      <c r="B38" s="32">
         <v>4.08</v>
       </c>
-      <c r="C38" s="31">
+      <c r="C38" s="32">
         <v>3.41</v>
       </c>
-      <c r="D38" s="31">
+      <c r="D38" s="32">
         <v>3.07</v>
       </c>
-      <c r="E38" s="31">
+      <c r="E38" s="32">
         <v>4.28</v>
       </c>
-      <c r="F38" s="31">
+      <c r="F38" s="32">
         <v>4.37</v>
       </c>
-      <c r="G38" s="31">
+      <c r="G38" s="32">
         <v>4.37</v>
       </c>
-      <c r="H38" s="31">
+      <c r="H38" s="32">
         <v>3.49</v>
       </c>
-      <c r="I38" s="31">
+      <c r="I38" s="32">
         <v>3.88</v>
       </c>
-      <c r="J38" s="31">
+      <c r="J38" s="32">
         <v>3.37</v>
       </c>
-      <c r="K38" s="31">
+      <c r="K38" s="32">
         <v>4.02</v>
       </c>
-      <c r="L38" s="31">
+      <c r="L38" s="32">
         <v>3.03</v>
       </c>
-      <c r="M38" s="31">
+      <c r="M38" s="32">
         <v>3.91</v>
       </c>
-      <c r="N38" s="31">
+      <c r="N38" s="32">
         <v>2.96</v>
       </c>
-      <c r="O38" s="31">
+      <c r="O38" s="32">
         <v>2.3</v>
       </c>
-      <c r="P38" s="31">
+      <c r="P38" s="32">
         <v>2.44</v>
       </c>
-      <c r="Q38" s="31">
+      <c r="Q38" s="32">
         <v>2.19</v>
       </c>
-      <c r="R38" s="31">
+      <c r="R38" s="32">
         <v>1.83</v>
       </c>
-      <c r="S38" s="31">
+      <c r="S38" s="32">
         <v>1.98</v>
       </c>
-      <c r="T38" s="31">
+      <c r="T38" s="32">
         <v>3.59</v>
       </c>
-      <c r="U38" s="31">
+      <c r="U38" s="32">
         <v>2.15</v>
       </c>
     </row>
     <row r="39" ht="15.0" customHeight="1">
-      <c r="A39" s="28" t="s">
-        <v>367</v>
-      </c>
-      <c r="B39" s="31">
+      <c r="A39" s="29" t="s">
+        <v>368</v>
+      </c>
+      <c r="B39" s="32">
         <v>3.79</v>
       </c>
-      <c r="C39" s="31">
+      <c r="C39" s="32">
         <v>3.8</v>
       </c>
-      <c r="D39" s="31">
+      <c r="D39" s="32">
         <v>3.86</v>
       </c>
-      <c r="E39" s="31">
+      <c r="E39" s="32">
         <v>4.11</v>
       </c>
-      <c r="F39" s="31">
+      <c r="F39" s="32">
         <v>3.94</v>
       </c>
-      <c r="G39" s="31">
+      <c r="G39" s="32">
         <v>3.85</v>
       </c>
-      <c r="H39" s="31">
+      <c r="H39" s="32">
         <v>3.57</v>
       </c>
-      <c r="I39" s="31">
+      <c r="I39" s="32">
         <v>3.64</v>
       </c>
-      <c r="J39" s="31">
+      <c r="J39" s="32">
         <v>3.48</v>
       </c>
-      <c r="K39" s="31">
+      <c r="K39" s="32">
         <v>3.34</v>
       </c>
-      <c r="L39" s="31">
+      <c r="L39" s="32">
         <v>2.98</v>
       </c>
-      <c r="M39" s="31">
+      <c r="M39" s="32">
         <v>2.84</v>
       </c>
-      <c r="N39" s="31">
+      <c r="N39" s="32">
         <v>2.4</v>
       </c>
-      <c r="O39" s="31">
+      <c r="O39" s="32">
         <v>2.18</v>
       </c>
-      <c r="P39" s="31">
+      <c r="P39" s="32">
         <v>2.39</v>
       </c>
-      <c r="Q39" s="31">
+      <c r="Q39" s="32">
         <v>2.32</v>
       </c>
-      <c r="R39" s="29"/>
-      <c r="S39" s="29"/>
-      <c r="T39" s="29"/>
-      <c r="U39" s="29"/>
+      <c r="R39" s="30"/>
+      <c r="S39" s="30"/>
+      <c r="T39" s="30"/>
+      <c r="U39" s="30"/>
     </row>
     <row r="40" ht="15.0" customHeight="1">
-      <c r="A40" s="26" t="s">
-        <v>368</v>
-      </c>
-      <c r="B40" s="27"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="27"/>
-      <c r="H40" s="27"/>
-      <c r="I40" s="27"/>
-      <c r="J40" s="27"/>
-      <c r="K40" s="27"/>
-      <c r="L40" s="27"/>
-      <c r="M40" s="27"/>
-      <c r="N40" s="27"/>
-      <c r="O40" s="27"/>
-      <c r="P40" s="27"/>
-      <c r="Q40" s="27"/>
-      <c r="R40" s="27"/>
-      <c r="S40" s="27"/>
-      <c r="T40" s="27"/>
-      <c r="U40" s="27"/>
+      <c r="A40" s="27" t="s">
+        <v>369</v>
+      </c>
+      <c r="B40" s="28"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="28"/>
+      <c r="G40" s="28"/>
+      <c r="H40" s="28"/>
+      <c r="I40" s="28"/>
+      <c r="J40" s="28"/>
+      <c r="K40" s="28"/>
+      <c r="L40" s="28"/>
+      <c r="M40" s="28"/>
+      <c r="N40" s="28"/>
+      <c r="O40" s="28"/>
+      <c r="P40" s="28"/>
+      <c r="Q40" s="28"/>
+      <c r="R40" s="28"/>
+      <c r="S40" s="28"/>
+      <c r="T40" s="28"/>
+      <c r="U40" s="28"/>
     </row>
     <row r="41" ht="15.0" customHeight="1">
-      <c r="A41" s="28" t="s">
-        <v>369</v>
-      </c>
-      <c r="B41" s="31">
+      <c r="A41" s="29" t="s">
+        <v>370</v>
+      </c>
+      <c r="B41" s="32">
         <v>4.7</v>
       </c>
-      <c r="C41" s="31">
+      <c r="C41" s="32">
         <v>4.13</v>
       </c>
-      <c r="D41" s="31">
+      <c r="D41" s="32">
         <v>3.78</v>
       </c>
-      <c r="E41" s="31">
+      <c r="E41" s="32">
         <v>5.48</v>
       </c>
-      <c r="F41" s="31">
+      <c r="F41" s="32">
         <v>5.82</v>
       </c>
-      <c r="G41" s="31">
+      <c r="G41" s="32">
         <v>5.75</v>
       </c>
-      <c r="H41" s="31">
+      <c r="H41" s="32">
         <v>4.51</v>
       </c>
-      <c r="I41" s="31">
+      <c r="I41" s="32">
         <v>5.2</v>
       </c>
-      <c r="J41" s="31">
+      <c r="J41" s="32">
         <v>4.63</v>
       </c>
-      <c r="K41" s="31">
+      <c r="K41" s="32">
         <v>5.7</v>
       </c>
-      <c r="L41" s="31">
+      <c r="L41" s="32">
         <v>4.05</v>
       </c>
-      <c r="M41" s="31">
+      <c r="M41" s="32">
         <v>5.48</v>
       </c>
-      <c r="N41" s="31">
+      <c r="N41" s="32">
         <v>4.21</v>
       </c>
-      <c r="O41" s="31">
+      <c r="O41" s="32">
         <v>3.0</v>
       </c>
-      <c r="P41" s="31">
+      <c r="P41" s="32">
         <v>3.11</v>
       </c>
-      <c r="Q41" s="31">
+      <c r="Q41" s="32">
         <v>2.97</v>
       </c>
-      <c r="R41" s="31">
+      <c r="R41" s="32">
         <v>2.81</v>
       </c>
-      <c r="S41" s="31">
+      <c r="S41" s="32">
         <v>2.85</v>
       </c>
-      <c r="T41" s="31">
+      <c r="T41" s="32">
         <v>4.98</v>
       </c>
-      <c r="U41" s="31">
+      <c r="U41" s="32">
         <v>2.58</v>
       </c>
     </row>
     <row r="42" ht="15.0" customHeight="1">
-      <c r="A42" s="28" t="s">
-        <v>370</v>
-      </c>
-      <c r="B42" s="31">
+      <c r="A42" s="29" t="s">
+        <v>371</v>
+      </c>
+      <c r="B42" s="32">
         <v>4.64</v>
       </c>
-      <c r="C42" s="31">
+      <c r="C42" s="32">
         <v>4.79</v>
       </c>
-      <c r="D42" s="31">
+      <c r="D42" s="32">
         <v>4.96</v>
       </c>
-      <c r="E42" s="31">
+      <c r="E42" s="32">
         <v>5.38</v>
       </c>
-      <c r="F42" s="31">
+      <c r="F42" s="32">
         <v>5.23</v>
       </c>
-      <c r="G42" s="31">
+      <c r="G42" s="32">
         <v>5.16</v>
       </c>
-      <c r="H42" s="31">
+      <c r="H42" s="32">
         <v>4.81</v>
       </c>
-      <c r="I42" s="31">
+      <c r="I42" s="32">
         <v>4.99</v>
       </c>
-      <c r="J42" s="31">
+      <c r="J42" s="32">
         <v>4.83</v>
       </c>
-      <c r="K42" s="31">
+      <c r="K42" s="32">
         <v>4.6</v>
       </c>
-      <c r="L42" s="31">
+      <c r="L42" s="32">
         <v>4.03</v>
       </c>
-      <c r="M42" s="31">
+      <c r="M42" s="32">
         <v>3.84</v>
       </c>
-      <c r="N42" s="31">
+      <c r="N42" s="32">
         <v>3.27</v>
       </c>
-      <c r="O42" s="31">
+      <c r="O42" s="32">
         <v>2.97</v>
       </c>
-      <c r="P42" s="31">
+      <c r="P42" s="32">
         <v>3.3</v>
       </c>
-      <c r="Q42" s="31">
+      <c r="Q42" s="32">
         <v>3.14</v>
       </c>
-      <c r="R42" s="29"/>
-      <c r="S42" s="29"/>
-      <c r="T42" s="29"/>
-      <c r="U42" s="29"/>
+      <c r="R42" s="30"/>
+      <c r="S42" s="30"/>
+      <c r="T42" s="30"/>
+      <c r="U42" s="30"/>
     </row>
     <row r="43" ht="15.0" customHeight="1">
-      <c r="A43" s="26" t="s">
-        <v>371</v>
-      </c>
-      <c r="B43" s="27"/>
-      <c r="C43" s="27"/>
-      <c r="D43" s="27"/>
-      <c r="E43" s="27"/>
-      <c r="F43" s="27"/>
-      <c r="G43" s="27"/>
-      <c r="H43" s="27"/>
-      <c r="I43" s="27"/>
-      <c r="J43" s="27"/>
-      <c r="K43" s="27"/>
-      <c r="L43" s="27"/>
-      <c r="M43" s="27"/>
-      <c r="N43" s="27"/>
-      <c r="O43" s="27"/>
-      <c r="P43" s="27"/>
-      <c r="Q43" s="27"/>
-      <c r="R43" s="27"/>
-      <c r="S43" s="27"/>
-      <c r="T43" s="27"/>
-      <c r="U43" s="27"/>
+      <c r="A43" s="27" t="s">
+        <v>372</v>
+      </c>
+      <c r="B43" s="28"/>
+      <c r="C43" s="28"/>
+      <c r="D43" s="28"/>
+      <c r="E43" s="28"/>
+      <c r="F43" s="28"/>
+      <c r="G43" s="28"/>
+      <c r="H43" s="28"/>
+      <c r="I43" s="28"/>
+      <c r="J43" s="28"/>
+      <c r="K43" s="28"/>
+      <c r="L43" s="28"/>
+      <c r="M43" s="28"/>
+      <c r="N43" s="28"/>
+      <c r="O43" s="28"/>
+      <c r="P43" s="28"/>
+      <c r="Q43" s="28"/>
+      <c r="R43" s="28"/>
+      <c r="S43" s="28"/>
+      <c r="T43" s="28"/>
+      <c r="U43" s="28"/>
     </row>
     <row r="44" ht="15.0" customHeight="1">
-      <c r="A44" s="28" t="s">
-        <v>372</v>
-      </c>
-      <c r="B44" s="31">
+      <c r="A44" s="29" t="s">
+        <v>373</v>
+      </c>
+      <c r="B44" s="32">
         <v>1.83</v>
       </c>
-      <c r="C44" s="31">
+      <c r="C44" s="32">
         <v>1.27</v>
       </c>
-      <c r="D44" s="31">
+      <c r="D44" s="32">
         <v>0.91</v>
       </c>
-      <c r="E44" s="31">
+      <c r="E44" s="32">
         <v>1.42</v>
       </c>
-      <c r="F44" s="31">
+      <c r="F44" s="32">
         <v>1.51</v>
       </c>
-      <c r="G44" s="31">
+      <c r="G44" s="32">
         <v>1.58</v>
       </c>
-      <c r="H44" s="31">
+      <c r="H44" s="32">
         <v>1.13</v>
       </c>
-      <c r="I44" s="31">
+      <c r="I44" s="32">
         <v>1.12</v>
       </c>
-      <c r="J44" s="31">
+      <c r="J44" s="32">
         <v>1.15</v>
       </c>
-      <c r="K44" s="31">
+      <c r="K44" s="32">
         <v>1.31</v>
       </c>
-      <c r="L44" s="31">
+      <c r="L44" s="32">
         <v>0.97</v>
       </c>
-      <c r="M44" s="31">
+      <c r="M44" s="32">
         <v>1.03</v>
       </c>
-      <c r="N44" s="31">
+      <c r="N44" s="32">
         <v>0.69</v>
       </c>
-      <c r="O44" s="31">
+      <c r="O44" s="32">
         <v>0.49</v>
       </c>
-      <c r="P44" s="31">
+      <c r="P44" s="32">
         <v>0.52</v>
       </c>
-      <c r="Q44" s="31">
+      <c r="Q44" s="32">
         <v>0.4</v>
       </c>
-      <c r="R44" s="31">
+      <c r="R44" s="32">
         <v>0.25</v>
       </c>
-      <c r="S44" s="31">
+      <c r="S44" s="32">
         <v>0.37</v>
       </c>
-      <c r="T44" s="31">
+      <c r="T44" s="32">
         <v>0.75</v>
       </c>
-      <c r="U44" s="29"/>
+      <c r="U44" s="30"/>
     </row>
     <row r="45" ht="15.0" customHeight="1">
-      <c r="A45" s="28" t="s">
-        <v>373</v>
-      </c>
-      <c r="B45" s="31">
+      <c r="A45" s="29" t="s">
+        <v>374</v>
+      </c>
+      <c r="B45" s="32">
         <v>1.36</v>
       </c>
-      <c r="C45" s="31">
+      <c r="C45" s="32">
         <v>1.29</v>
       </c>
-      <c r="D45" s="31">
+      <c r="D45" s="32">
         <v>1.27</v>
       </c>
-      <c r="E45" s="31">
+      <c r="E45" s="32">
         <v>1.36</v>
       </c>
-      <c r="F45" s="31">
+      <c r="F45" s="32">
         <v>1.31</v>
       </c>
-      <c r="G45" s="31">
+      <c r="G45" s="32">
         <v>1.27</v>
       </c>
-      <c r="H45" s="31">
+      <c r="H45" s="32">
         <v>1.14</v>
       </c>
-      <c r="I45" s="31">
+      <c r="I45" s="32">
         <v>1.13</v>
       </c>
-      <c r="J45" s="31">
+      <c r="J45" s="32">
         <v>1.05</v>
       </c>
-      <c r="K45" s="31">
+      <c r="K45" s="32">
         <v>0.91</v>
       </c>
-      <c r="L45" s="31">
+      <c r="L45" s="32">
         <v>0.75</v>
       </c>
-      <c r="M45" s="31">
+      <c r="M45" s="32">
         <v>0.63</v>
       </c>
-      <c r="N45" s="31">
+      <c r="N45" s="32">
         <v>0.47</v>
       </c>
-      <c r="O45" s="31">
+      <c r="O45" s="32">
         <v>0.4</v>
       </c>
-      <c r="P45" s="31">
+      <c r="P45" s="32">
         <v>0.44</v>
       </c>
-      <c r="Q45" s="29"/>
-      <c r="R45" s="29"/>
-      <c r="S45" s="29"/>
-      <c r="T45" s="29"/>
-      <c r="U45" s="29"/>
+      <c r="Q45" s="30"/>
+      <c r="R45" s="30"/>
+      <c r="S45" s="30"/>
+      <c r="T45" s="30"/>
+      <c r="U45" s="30"/>
     </row>
     <row r="46" ht="15.0" customHeight="1">
-      <c r="A46" s="26" t="s">
-        <v>374</v>
-      </c>
-      <c r="B46" s="27"/>
-      <c r="C46" s="27"/>
-      <c r="D46" s="27"/>
-      <c r="E46" s="27"/>
-      <c r="F46" s="27"/>
-      <c r="G46" s="27"/>
-      <c r="H46" s="27"/>
-      <c r="I46" s="27"/>
-      <c r="J46" s="27"/>
-      <c r="K46" s="27"/>
-      <c r="L46" s="27"/>
-      <c r="M46" s="27"/>
-      <c r="N46" s="27"/>
-      <c r="O46" s="27"/>
-      <c r="P46" s="27"/>
-      <c r="Q46" s="27"/>
-      <c r="R46" s="27"/>
-      <c r="S46" s="27"/>
-      <c r="T46" s="27"/>
-      <c r="U46" s="27"/>
+      <c r="A46" s="27" t="s">
+        <v>375</v>
+      </c>
+      <c r="B46" s="28"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="28"/>
+      <c r="E46" s="28"/>
+      <c r="F46" s="28"/>
+      <c r="G46" s="28"/>
+      <c r="H46" s="28"/>
+      <c r="I46" s="28"/>
+      <c r="J46" s="28"/>
+      <c r="K46" s="28"/>
+      <c r="L46" s="28"/>
+      <c r="M46" s="28"/>
+      <c r="N46" s="28"/>
+      <c r="O46" s="28"/>
+      <c r="P46" s="28"/>
+      <c r="Q46" s="28"/>
+      <c r="R46" s="28"/>
+      <c r="S46" s="28"/>
+      <c r="T46" s="28"/>
+      <c r="U46" s="28"/>
     </row>
     <row r="47" ht="15.0" customHeight="1">
-      <c r="A47" s="28" t="s">
-        <v>375</v>
-      </c>
-      <c r="B47" s="31">
+      <c r="A47" s="29" t="s">
+        <v>376</v>
+      </c>
+      <c r="B47" s="32">
         <v>74.29</v>
       </c>
-      <c r="C47" s="31">
+      <c r="C47" s="32">
         <v>14.34</v>
       </c>
-      <c r="D47" s="29"/>
-      <c r="E47" s="29"/>
-      <c r="F47" s="31">
+      <c r="D47" s="30"/>
+      <c r="E47" s="30"/>
+      <c r="F47" s="32">
         <v>32.91</v>
       </c>
-      <c r="G47" s="31">
+      <c r="G47" s="32">
         <v>59.66</v>
       </c>
-      <c r="H47" s="31">
+      <c r="H47" s="32">
         <v>85.3</v>
       </c>
-      <c r="I47" s="30">
+      <c r="I47" s="31">
         <v>105.34</v>
       </c>
-      <c r="J47" s="30">
+      <c r="J47" s="31">
         <v>107.42</v>
       </c>
-      <c r="K47" s="31">
+      <c r="K47" s="32">
         <v>35.59</v>
       </c>
-      <c r="L47" s="30">
+      <c r="L47" s="31">
         <v>186.52</v>
       </c>
-      <c r="M47" s="31">
+      <c r="M47" s="32">
         <v>22.97</v>
       </c>
-      <c r="N47" s="31">
+      <c r="N47" s="32">
         <v>9.99</v>
       </c>
-      <c r="O47" s="29"/>
-      <c r="P47" s="31">
+      <c r="O47" s="30"/>
+      <c r="P47" s="32">
         <v>18.27</v>
       </c>
-      <c r="Q47" s="31">
+      <c r="Q47" s="32">
         <v>3.29</v>
       </c>
-      <c r="R47" s="29"/>
-      <c r="S47" s="29"/>
-      <c r="T47" s="29"/>
-      <c r="U47" s="29"/>
+      <c r="R47" s="30"/>
+      <c r="S47" s="30"/>
+      <c r="T47" s="30"/>
+      <c r="U47" s="30"/>
     </row>
     <row r="48" ht="15.0" customHeight="1">
-      <c r="A48" s="28" t="s">
-        <v>376</v>
-      </c>
-      <c r="B48" s="31">
+      <c r="A48" s="29" t="s">
+        <v>377</v>
+      </c>
+      <c r="B48" s="32">
         <v>55.3</v>
       </c>
-      <c r="C48" s="31">
+      <c r="C48" s="32">
         <v>51.6</v>
       </c>
-      <c r="D48" s="30">
+      <c r="D48" s="31">
         <v>209.03</v>
       </c>
-      <c r="E48" s="31">
+      <c r="E48" s="32">
         <v>76.78</v>
       </c>
-      <c r="F48" s="31">
+      <c r="F48" s="32">
         <v>59.41</v>
       </c>
-      <c r="G48" s="31">
+      <c r="G48" s="32">
         <v>66.18</v>
       </c>
-      <c r="H48" s="31">
+      <c r="H48" s="32">
         <v>75.66</v>
       </c>
-      <c r="I48" s="31">
+      <c r="I48" s="32">
         <v>55.12</v>
       </c>
-      <c r="J48" s="31">
+      <c r="J48" s="32">
         <v>32.84</v>
       </c>
-      <c r="K48" s="31">
+      <c r="K48" s="32">
         <v>39.47</v>
       </c>
-      <c r="L48" s="31">
+      <c r="L48" s="32">
         <v>35.86</v>
       </c>
-      <c r="M48" s="31">
+      <c r="M48" s="32">
         <v>14.16</v>
       </c>
-      <c r="N48" s="31">
+      <c r="N48" s="32">
         <v>15.45</v>
       </c>
-      <c r="O48" s="31">
+      <c r="O48" s="32">
         <v>91.31</v>
       </c>
-      <c r="P48" s="31">
+      <c r="P48" s="32">
         <v>43.09</v>
       </c>
-      <c r="Q48" s="29"/>
-      <c r="R48" s="29"/>
-      <c r="S48" s="29"/>
-      <c r="T48" s="29"/>
-      <c r="U48" s="29"/>
+      <c r="Q48" s="30"/>
+      <c r="R48" s="30"/>
+      <c r="S48" s="30"/>
+      <c r="T48" s="30"/>
+      <c r="U48" s="30"/>
     </row>
     <row r="49" ht="15.0" customHeight="1">
-      <c r="A49" s="26" t="s">
-        <v>377</v>
-      </c>
-      <c r="B49" s="27"/>
-      <c r="C49" s="27"/>
-      <c r="D49" s="27"/>
-      <c r="E49" s="27"/>
-      <c r="F49" s="27"/>
-      <c r="G49" s="27"/>
-      <c r="H49" s="27"/>
-      <c r="I49" s="27"/>
-      <c r="J49" s="27"/>
-      <c r="K49" s="27"/>
-      <c r="L49" s="27"/>
-      <c r="M49" s="27"/>
-      <c r="N49" s="27"/>
-      <c r="O49" s="27"/>
-      <c r="P49" s="27"/>
-      <c r="Q49" s="27"/>
-      <c r="R49" s="27"/>
-      <c r="S49" s="27"/>
-      <c r="T49" s="27"/>
-      <c r="U49" s="27"/>
+      <c r="A49" s="27" t="s">
+        <v>378</v>
+      </c>
+      <c r="B49" s="28"/>
+      <c r="C49" s="28"/>
+      <c r="D49" s="28"/>
+      <c r="E49" s="28"/>
+      <c r="F49" s="28"/>
+      <c r="G49" s="28"/>
+      <c r="H49" s="28"/>
+      <c r="I49" s="28"/>
+      <c r="J49" s="28"/>
+      <c r="K49" s="28"/>
+      <c r="L49" s="28"/>
+      <c r="M49" s="28"/>
+      <c r="N49" s="28"/>
+      <c r="O49" s="28"/>
+      <c r="P49" s="28"/>
+      <c r="Q49" s="28"/>
+      <c r="R49" s="28"/>
+      <c r="S49" s="28"/>
+      <c r="T49" s="28"/>
+      <c r="U49" s="28"/>
     </row>
     <row r="50" ht="15.0" customHeight="1">
-      <c r="A50" s="28" t="s">
-        <v>378</v>
-      </c>
-      <c r="B50" s="31">
+      <c r="A50" s="29" t="s">
+        <v>379</v>
+      </c>
+      <c r="B50" s="32">
         <v>18.67</v>
       </c>
-      <c r="C50" s="31">
+      <c r="C50" s="32">
         <v>15.31</v>
       </c>
-      <c r="D50" s="31">
+      <c r="D50" s="32">
         <v>17.91</v>
       </c>
-      <c r="E50" s="31">
+      <c r="E50" s="32">
         <v>23.24</v>
       </c>
-      <c r="F50" s="31">
+      <c r="F50" s="32">
         <v>18.26</v>
       </c>
-      <c r="G50" s="31">
+      <c r="G50" s="32">
         <v>20.53</v>
       </c>
-      <c r="H50" s="31">
+      <c r="H50" s="32">
         <v>16.45</v>
       </c>
-      <c r="I50" s="31">
+      <c r="I50" s="32">
         <v>17.44</v>
       </c>
-      <c r="J50" s="31">
+      <c r="J50" s="32">
         <v>16.86</v>
       </c>
-      <c r="K50" s="31">
+      <c r="K50" s="32">
         <v>19.19</v>
       </c>
-      <c r="L50" s="31">
+      <c r="L50" s="32">
         <v>13.68</v>
       </c>
-      <c r="M50" s="31">
+      <c r="M50" s="32">
         <v>15.79</v>
       </c>
-      <c r="N50" s="31">
+      <c r="N50" s="32">
         <v>11.71</v>
       </c>
-      <c r="O50" s="31">
+      <c r="O50" s="32">
         <v>8.55</v>
       </c>
-      <c r="P50" s="31">
+      <c r="P50" s="32">
         <v>7.69</v>
       </c>
-      <c r="Q50" s="31">
+      <c r="Q50" s="32">
         <v>5.15</v>
       </c>
-      <c r="R50" s="31">
+      <c r="R50" s="32">
         <v>11.68</v>
       </c>
-      <c r="S50" s="31">
+      <c r="S50" s="32">
         <v>6.79</v>
       </c>
-      <c r="T50" s="31">
+      <c r="T50" s="32">
         <v>16.98</v>
       </c>
-      <c r="U50" s="29"/>
+      <c r="U50" s="30"/>
     </row>
     <row r="51" ht="15.0" customHeight="1">
-      <c r="A51" s="28" t="s">
-        <v>379</v>
-      </c>
-      <c r="B51" s="31">
+      <c r="A51" s="29" t="s">
+        <v>380</v>
+      </c>
+      <c r="B51" s="32">
         <v>18.3</v>
       </c>
-      <c r="C51" s="31">
+      <c r="C51" s="32">
         <v>18.55</v>
       </c>
-      <c r="D51" s="31">
+      <c r="D51" s="32">
         <v>19.29</v>
       </c>
-      <c r="E51" s="31">
+      <c r="E51" s="32">
         <v>19.32</v>
       </c>
-      <c r="F51" s="31">
+      <c r="F51" s="32">
         <v>18.06</v>
       </c>
-      <c r="G51" s="31">
+      <c r="G51" s="32">
         <v>18.19</v>
       </c>
-      <c r="H51" s="31">
+      <c r="H51" s="32">
         <v>16.77</v>
       </c>
-      <c r="I51" s="31">
+      <c r="I51" s="32">
         <v>16.71</v>
       </c>
-      <c r="J51" s="31">
+      <c r="J51" s="32">
         <v>15.71</v>
       </c>
-      <c r="K51" s="31">
+      <c r="K51" s="32">
         <v>14.19</v>
       </c>
-      <c r="L51" s="31">
+      <c r="L51" s="32">
         <v>11.67</v>
       </c>
-      <c r="M51" s="31">
+      <c r="M51" s="32">
         <v>9.64</v>
       </c>
-      <c r="N51" s="31">
+      <c r="N51" s="32">
         <v>8.36</v>
       </c>
-      <c r="O51" s="31">
+      <c r="O51" s="32">
         <v>7.34</v>
       </c>
-      <c r="P51" s="31">
+      <c r="P51" s="32">
         <v>8.26</v>
       </c>
-      <c r="Q51" s="29"/>
-      <c r="R51" s="29"/>
-      <c r="S51" s="29"/>
-      <c r="T51" s="29"/>
-      <c r="U51" s="29"/>
+      <c r="Q51" s="30"/>
+      <c r="R51" s="30"/>
+      <c r="S51" s="30"/>
+      <c r="T51" s="30"/>
+      <c r="U51" s="30"/>
     </row>
     <row r="52" ht="15.0" customHeight="1">
-      <c r="A52" s="26" t="s">
-        <v>380</v>
-      </c>
-      <c r="B52" s="27"/>
-      <c r="C52" s="27"/>
-      <c r="D52" s="27"/>
-      <c r="E52" s="27"/>
-      <c r="F52" s="27"/>
-      <c r="G52" s="27"/>
-      <c r="H52" s="27"/>
-      <c r="I52" s="27"/>
-      <c r="J52" s="27"/>
-      <c r="K52" s="27"/>
-      <c r="L52" s="27"/>
-      <c r="M52" s="27"/>
-      <c r="N52" s="27"/>
-      <c r="O52" s="27"/>
-      <c r="P52" s="27"/>
-      <c r="Q52" s="27"/>
-      <c r="R52" s="27"/>
-      <c r="S52" s="27"/>
-      <c r="T52" s="27"/>
-      <c r="U52" s="27"/>
+      <c r="A52" s="27" t="s">
+        <v>381</v>
+      </c>
+      <c r="B52" s="28"/>
+      <c r="C52" s="28"/>
+      <c r="D52" s="28"/>
+      <c r="E52" s="28"/>
+      <c r="F52" s="28"/>
+      <c r="G52" s="28"/>
+      <c r="H52" s="28"/>
+      <c r="I52" s="28"/>
+      <c r="J52" s="28"/>
+      <c r="K52" s="28"/>
+      <c r="L52" s="28"/>
+      <c r="M52" s="28"/>
+      <c r="N52" s="28"/>
+      <c r="O52" s="28"/>
+      <c r="P52" s="28"/>
+      <c r="Q52" s="28"/>
+      <c r="R52" s="28"/>
+      <c r="S52" s="28"/>
+      <c r="T52" s="28"/>
+      <c r="U52" s="28"/>
     </row>
     <row r="53" ht="15.0" customHeight="1">
-      <c r="A53" s="28" t="s">
-        <v>381</v>
-      </c>
-      <c r="B53" s="31">
+      <c r="A53" s="29" t="s">
+        <v>382</v>
+      </c>
+      <c r="B53" s="32">
         <v>23.26</v>
       </c>
-      <c r="C53" s="31">
+      <c r="C53" s="32">
         <v>19.8</v>
       </c>
-      <c r="D53" s="31">
+      <c r="D53" s="32">
         <v>26.01</v>
       </c>
-      <c r="E53" s="31">
+      <c r="E53" s="32">
         <v>35.02</v>
       </c>
-      <c r="F53" s="31">
+      <c r="F53" s="32">
         <v>26.97</v>
       </c>
-      <c r="G53" s="31">
+      <c r="G53" s="32">
         <v>30.37</v>
       </c>
-      <c r="H53" s="31">
+      <c r="H53" s="32">
         <v>23.55</v>
       </c>
-      <c r="I53" s="31">
+      <c r="I53" s="32">
         <v>24.88</v>
       </c>
-      <c r="J53" s="31">
+      <c r="J53" s="32">
         <v>25.28</v>
       </c>
-      <c r="K53" s="31">
+      <c r="K53" s="32">
         <v>28.3</v>
       </c>
-      <c r="L53" s="31">
+      <c r="L53" s="32">
         <v>19.73</v>
       </c>
-      <c r="M53" s="31">
+      <c r="M53" s="32">
         <v>23.38</v>
       </c>
-      <c r="N53" s="31">
+      <c r="N53" s="32">
         <v>18.18</v>
       </c>
-      <c r="O53" s="31">
+      <c r="O53" s="32">
         <v>13.55</v>
       </c>
-      <c r="P53" s="31">
+      <c r="P53" s="32">
         <v>12.35</v>
       </c>
-      <c r="Q53" s="31">
+      <c r="Q53" s="32">
         <v>7.77</v>
       </c>
-      <c r="R53" s="30">
+      <c r="R53" s="31">
         <v>4330.07</v>
       </c>
-      <c r="S53" s="31">
+      <c r="S53" s="32">
         <v>15.22</v>
       </c>
-      <c r="T53" s="31">
+      <c r="T53" s="32">
         <v>47.96</v>
       </c>
-      <c r="U53" s="29"/>
+      <c r="U53" s="30"/>
     </row>
     <row r="54" ht="15.0" customHeight="1">
-      <c r="A54" s="28" t="s">
-        <v>382</v>
-      </c>
-      <c r="B54" s="31">
+      <c r="A54" s="29" t="s">
+        <v>383</v>
+      </c>
+      <c r="B54" s="32">
         <v>24.82</v>
       </c>
-      <c r="C54" s="31">
+      <c r="C54" s="32">
         <v>26.32</v>
       </c>
-      <c r="D54" s="31">
+      <c r="D54" s="32">
         <v>28.34</v>
       </c>
-      <c r="E54" s="31">
+      <c r="E54" s="32">
         <v>28.32</v>
       </c>
-      <c r="F54" s="31">
+      <c r="F54" s="32">
         <v>26.41</v>
       </c>
-      <c r="G54" s="31">
+      <c r="G54" s="32">
         <v>26.56</v>
       </c>
-      <c r="H54" s="31">
+      <c r="H54" s="32">
         <v>24.36</v>
       </c>
-      <c r="I54" s="31">
+      <c r="I54" s="32">
         <v>24.44</v>
       </c>
-      <c r="J54" s="31">
+      <c r="J54" s="32">
         <v>23.36</v>
       </c>
-      <c r="K54" s="31">
+      <c r="K54" s="32">
         <v>21.27</v>
       </c>
-      <c r="L54" s="31">
+      <c r="L54" s="32">
         <v>17.79</v>
       </c>
-      <c r="M54" s="31">
+      <c r="M54" s="32">
         <v>14.86</v>
       </c>
-      <c r="N54" s="31">
+      <c r="N54" s="32">
         <v>14.18</v>
       </c>
-      <c r="O54" s="31">
+      <c r="O54" s="32">
         <v>13.27</v>
       </c>
-      <c r="P54" s="31">
+      <c r="P54" s="32">
         <v>16.25</v>
       </c>
-      <c r="Q54" s="29"/>
-      <c r="R54" s="29"/>
-      <c r="S54" s="29"/>
-      <c r="T54" s="29"/>
-      <c r="U54" s="29"/>
+      <c r="Q54" s="30"/>
+      <c r="R54" s="30"/>
+      <c r="S54" s="30"/>
+      <c r="T54" s="30"/>
+      <c r="U54" s="30"/>
     </row>
     <row r="55" ht="15.0" customHeight="1">
-      <c r="A55" s="26" t="s">
-        <v>383</v>
-      </c>
-      <c r="B55" s="27"/>
-      <c r="C55" s="27"/>
-      <c r="D55" s="27"/>
-      <c r="E55" s="27"/>
-      <c r="F55" s="27"/>
-      <c r="G55" s="27"/>
-      <c r="H55" s="27"/>
-      <c r="I55" s="27"/>
-      <c r="J55" s="27"/>
-      <c r="K55" s="27"/>
-      <c r="L55" s="27"/>
-      <c r="M55" s="27"/>
-      <c r="N55" s="27"/>
-      <c r="O55" s="27"/>
-      <c r="P55" s="27"/>
-      <c r="Q55" s="27"/>
-      <c r="R55" s="27"/>
-      <c r="S55" s="27"/>
-      <c r="T55" s="27"/>
-      <c r="U55" s="27"/>
+      <c r="A55" s="27" t="s">
+        <v>384</v>
+      </c>
+      <c r="B55" s="28"/>
+      <c r="C55" s="28"/>
+      <c r="D55" s="28"/>
+      <c r="E55" s="28"/>
+      <c r="F55" s="28"/>
+      <c r="G55" s="28"/>
+      <c r="H55" s="28"/>
+      <c r="I55" s="28"/>
+      <c r="J55" s="28"/>
+      <c r="K55" s="28"/>
+      <c r="L55" s="28"/>
+      <c r="M55" s="28"/>
+      <c r="N55" s="28"/>
+      <c r="O55" s="28"/>
+      <c r="P55" s="28"/>
+      <c r="Q55" s="28"/>
+      <c r="R55" s="28"/>
+      <c r="S55" s="28"/>
+      <c r="T55" s="28"/>
+      <c r="U55" s="28"/>
     </row>
     <row r="56" ht="15.0" customHeight="1">
-      <c r="A56" s="28" t="s">
-        <v>384</v>
-      </c>
-      <c r="B56" s="31">
+      <c r="A56" s="29" t="s">
+        <v>385</v>
+      </c>
+      <c r="B56" s="32">
         <v>22.86</v>
       </c>
-      <c r="C56" s="31">
+      <c r="C56" s="32">
         <v>19.31</v>
       </c>
-      <c r="D56" s="31">
+      <c r="D56" s="32">
         <v>21.64</v>
       </c>
-      <c r="E56" s="31">
+      <c r="E56" s="32">
         <v>25.39</v>
       </c>
-      <c r="F56" s="31">
+      <c r="F56" s="32">
         <v>26.51</v>
       </c>
-      <c r="G56" s="31">
+      <c r="G56" s="32">
         <v>30.37</v>
       </c>
-      <c r="H56" s="31">
+      <c r="H56" s="32">
         <v>23.55</v>
       </c>
-      <c r="I56" s="31">
+      <c r="I56" s="32">
         <v>24.88</v>
       </c>
-      <c r="J56" s="31">
+      <c r="J56" s="32">
         <v>24.9</v>
       </c>
-      <c r="K56" s="31">
+      <c r="K56" s="32">
         <v>29.7</v>
       </c>
-      <c r="L56" s="31">
+      <c r="L56" s="32">
         <v>22.3</v>
       </c>
-      <c r="M56" s="31">
+      <c r="M56" s="32">
         <v>23.38</v>
       </c>
-      <c r="N56" s="31">
+      <c r="N56" s="32">
         <v>18.18</v>
       </c>
-      <c r="O56" s="31">
+      <c r="O56" s="32">
         <v>13.33</v>
       </c>
-      <c r="P56" s="31">
+      <c r="P56" s="32">
         <v>12.35</v>
       </c>
-      <c r="Q56" s="31">
+      <c r="Q56" s="32">
         <v>7.77</v>
       </c>
-      <c r="R56" s="30">
+      <c r="R56" s="31">
         <v>4330.07</v>
       </c>
-      <c r="S56" s="31">
+      <c r="S56" s="32">
         <v>13.13</v>
       </c>
-      <c r="T56" s="31">
+      <c r="T56" s="32">
         <v>47.96</v>
       </c>
-      <c r="U56" s="29"/>
+      <c r="U56" s="30"/>
     </row>
     <row r="57" ht="15.0" customHeight="1">
-      <c r="A57" s="28" t="s">
-        <v>385</v>
-      </c>
-      <c r="B57" s="31">
+      <c r="A57" s="29" t="s">
+        <v>386</v>
+      </c>
+      <c r="B57" s="32">
         <v>3.79</v>
       </c>
-      <c r="C57" s="31">
+      <c r="C57" s="32">
         <v>3.8</v>
       </c>
-      <c r="D57" s="31">
+      <c r="D57" s="32">
         <v>3.86</v>
       </c>
-      <c r="E57" s="31">
+      <c r="E57" s="32">
         <v>4.11</v>
       </c>
-      <c r="F57" s="31">
+      <c r="F57" s="32">
         <v>3.94</v>
       </c>
-      <c r="G57" s="31">
+      <c r="G57" s="32">
         <v>3.85</v>
       </c>
-      <c r="H57" s="31">
+      <c r="H57" s="32">
         <v>3.57</v>
       </c>
-      <c r="I57" s="31">
+      <c r="I57" s="32">
         <v>3.64</v>
       </c>
-      <c r="J57" s="31">
+      <c r="J57" s="32">
         <v>3.48</v>
       </c>
-      <c r="K57" s="31">
+      <c r="K57" s="32">
         <v>3.34</v>
       </c>
-      <c r="L57" s="31">
+      <c r="L57" s="32">
         <v>2.98</v>
       </c>
-      <c r="M57" s="31">
+      <c r="M57" s="32">
         <v>2.84</v>
       </c>
-      <c r="N57" s="31">
+      <c r="N57" s="32">
         <v>2.4</v>
       </c>
-      <c r="O57" s="31">
+      <c r="O57" s="32">
         <v>2.18</v>
       </c>
-      <c r="P57" s="31">
+      <c r="P57" s="32">
         <v>2.39</v>
       </c>
-      <c r="Q57" s="31">
+      <c r="Q57" s="32">
         <v>2.32</v>
       </c>
-      <c r="R57" s="29"/>
-      <c r="S57" s="29"/>
-      <c r="T57" s="29"/>
-      <c r="U57" s="29"/>
+      <c r="R57" s="30"/>
+      <c r="S57" s="30"/>
+      <c r="T57" s="30"/>
+      <c r="U57" s="30"/>
     </row>
     <row r="58" ht="15.0" customHeight="1">
-      <c r="A58" s="26" t="s">
-        <v>386</v>
-      </c>
-      <c r="B58" s="27"/>
-      <c r="C58" s="27"/>
-      <c r="D58" s="27"/>
-      <c r="E58" s="27"/>
-      <c r="F58" s="27"/>
-      <c r="G58" s="27"/>
-      <c r="H58" s="27"/>
-      <c r="I58" s="27"/>
-      <c r="J58" s="27"/>
-      <c r="K58" s="27"/>
-      <c r="L58" s="27"/>
-      <c r="M58" s="27"/>
-      <c r="N58" s="27"/>
-      <c r="O58" s="27"/>
-      <c r="P58" s="27"/>
-      <c r="Q58" s="27"/>
-      <c r="R58" s="27"/>
-      <c r="S58" s="27"/>
-      <c r="T58" s="27"/>
-      <c r="U58" s="27"/>
+      <c r="A58" s="27" t="s">
+        <v>387</v>
+      </c>
+      <c r="B58" s="28"/>
+      <c r="C58" s="28"/>
+      <c r="D58" s="28"/>
+      <c r="E58" s="28"/>
+      <c r="F58" s="28"/>
+      <c r="G58" s="28"/>
+      <c r="H58" s="28"/>
+      <c r="I58" s="28"/>
+      <c r="J58" s="28"/>
+      <c r="K58" s="28"/>
+      <c r="L58" s="28"/>
+      <c r="M58" s="28"/>
+      <c r="N58" s="28"/>
+      <c r="O58" s="28"/>
+      <c r="P58" s="28"/>
+      <c r="Q58" s="28"/>
+      <c r="R58" s="28"/>
+      <c r="S58" s="28"/>
+      <c r="T58" s="28"/>
+      <c r="U58" s="28"/>
     </row>
     <row r="59" ht="15.0" customHeight="1">
-      <c r="A59" s="28" t="s">
-        <v>387</v>
-      </c>
-      <c r="B59" s="31">
+      <c r="A59" s="29" t="s">
+        <v>388</v>
+      </c>
+      <c r="B59" s="32">
         <v>1.19</v>
       </c>
-      <c r="C59" s="31">
+      <c r="C59" s="32">
         <v>0.3</v>
       </c>
-      <c r="D59" s="31">
+      <c r="D59" s="32">
         <v>1.15</v>
       </c>
-      <c r="E59" s="34">
+      <c r="E59" s="35">
         <v>-3.73</v>
       </c>
-      <c r="F59" s="31">
+      <c r="F59" s="32">
         <v>5.37</v>
       </c>
-      <c r="G59" s="31">
+      <c r="G59" s="32">
         <v>2.43</v>
       </c>
-      <c r="H59" s="31">
+      <c r="H59" s="32">
         <v>2.2</v>
       </c>
-      <c r="I59" s="31">
+      <c r="I59" s="32">
         <v>1.31</v>
       </c>
-      <c r="J59" s="31">
+      <c r="J59" s="32">
         <v>3.63</v>
       </c>
-      <c r="K59" s="31">
+      <c r="K59" s="32">
         <v>5.89</v>
       </c>
-      <c r="L59" s="31">
+      <c r="L59" s="32">
         <v>0.98</v>
       </c>
-      <c r="M59" s="31">
+      <c r="M59" s="32">
         <v>1.45</v>
       </c>
-      <c r="N59" s="31">
+      <c r="N59" s="32">
         <v>5.81</v>
       </c>
-      <c r="O59" s="34">
+      <c r="O59" s="35">
         <v>-3.84</v>
       </c>
-      <c r="P59" s="34">
+      <c r="P59" s="35">
         <v>-0.51</v>
       </c>
-      <c r="Q59" s="29">
+      <c r="Q59" s="30">
         <v>0.0</v>
       </c>
-      <c r="R59" s="34">
+      <c r="R59" s="35">
         <v>-43.44</v>
       </c>
-      <c r="S59" s="31">
+      <c r="S59" s="32">
         <v>0.18</v>
       </c>
-      <c r="T59" s="29"/>
-      <c r="U59" s="29"/>
+      <c r="T59" s="30"/>
+      <c r="U59" s="30"/>
     </row>
     <row r="60" ht="15.0" customHeight="1">
-      <c r="A60" s="28" t="s">
-        <v>388</v>
-      </c>
-      <c r="B60" s="31">
+      <c r="A60" s="29" t="s">
+        <v>389</v>
+      </c>
+      <c r="B60" s="32">
         <v>1.36</v>
       </c>
-      <c r="C60" s="31">
+      <c r="C60" s="32">
         <v>1.56</v>
       </c>
-      <c r="D60" s="31">
+      <c r="D60" s="32">
         <v>3.65</v>
       </c>
-      <c r="E60" s="31">
+      <c r="E60" s="32">
         <v>3.98</v>
       </c>
-      <c r="F60" s="31">
+      <c r="F60" s="32">
         <v>2.46</v>
       </c>
-      <c r="G60" s="31">
+      <c r="G60" s="32">
         <v>2.48</v>
       </c>
-      <c r="H60" s="31">
+      <c r="H60" s="32">
         <v>2.01</v>
       </c>
-      <c r="I60" s="31">
+      <c r="I60" s="32">
         <v>1.85</v>
       </c>
-      <c r="J60" s="31">
+      <c r="J60" s="32">
         <v>2.33</v>
       </c>
-      <c r="K60" s="31">
+      <c r="K60" s="32">
         <v>2.74</v>
       </c>
-      <c r="L60" s="31">
+      <c r="L60" s="32">
         <v>19.08</v>
       </c>
-      <c r="M60" s="31">
+      <c r="M60" s="32">
         <v>0.05</v>
       </c>
-      <c r="N60" s="31">
+      <c r="N60" s="32">
         <v>0.97</v>
       </c>
-      <c r="O60" s="31">
+      <c r="O60" s="32">
         <v>0.46</v>
       </c>
-      <c r="P60" s="29"/>
-      <c r="Q60" s="29"/>
-      <c r="R60" s="29"/>
-      <c r="S60" s="29"/>
-      <c r="T60" s="29"/>
-      <c r="U60" s="29"/>
+      <c r="P60" s="30"/>
+      <c r="Q60" s="30"/>
+      <c r="R60" s="30"/>
+      <c r="S60" s="30"/>
+      <c r="T60" s="30"/>
+      <c r="U60" s="30"/>
     </row>
     <row r="61" ht="15.0" customHeight="1">
-      <c r="A61" s="26" t="s">
-        <v>389</v>
-      </c>
-      <c r="B61" s="27"/>
-      <c r="C61" s="27"/>
-      <c r="D61" s="27"/>
-      <c r="E61" s="27"/>
-      <c r="F61" s="27"/>
-      <c r="G61" s="27"/>
-      <c r="H61" s="27"/>
-      <c r="I61" s="27"/>
-      <c r="J61" s="27"/>
-      <c r="K61" s="27"/>
-      <c r="L61" s="27"/>
-      <c r="M61" s="27"/>
-      <c r="N61" s="27"/>
-      <c r="O61" s="27"/>
-      <c r="P61" s="27"/>
-      <c r="Q61" s="27"/>
-      <c r="R61" s="27"/>
-      <c r="S61" s="27"/>
-      <c r="T61" s="27"/>
-      <c r="U61" s="27"/>
+      <c r="A61" s="27" t="s">
+        <v>390</v>
+      </c>
+      <c r="B61" s="28"/>
+      <c r="C61" s="28"/>
+      <c r="D61" s="28"/>
+      <c r="E61" s="28"/>
+      <c r="F61" s="28"/>
+      <c r="G61" s="28"/>
+      <c r="H61" s="28"/>
+      <c r="I61" s="28"/>
+      <c r="J61" s="28"/>
+      <c r="K61" s="28"/>
+      <c r="L61" s="28"/>
+      <c r="M61" s="28"/>
+      <c r="N61" s="28"/>
+      <c r="O61" s="28"/>
+      <c r="P61" s="28"/>
+      <c r="Q61" s="28"/>
+      <c r="R61" s="28"/>
+      <c r="S61" s="28"/>
+      <c r="T61" s="28"/>
+      <c r="U61" s="28"/>
     </row>
     <row r="62" ht="15.0" customHeight="1">
-      <c r="A62" s="28" t="s">
-        <v>390</v>
-      </c>
-      <c r="B62" s="31">
+      <c r="A62" s="29" t="s">
+        <v>391</v>
+      </c>
+      <c r="B62" s="32">
         <v>1.86</v>
       </c>
-      <c r="C62" s="31">
+      <c r="C62" s="32">
         <v>1.33</v>
       </c>
-      <c r="D62" s="31">
+      <c r="D62" s="32">
         <v>1.03</v>
       </c>
-      <c r="E62" s="31">
+      <c r="E62" s="32">
         <v>1.53</v>
       </c>
-      <c r="F62" s="31">
+      <c r="F62" s="32">
         <v>1.63</v>
       </c>
-      <c r="G62" s="31">
+      <c r="G62" s="32">
         <v>1.72</v>
       </c>
-      <c r="H62" s="31">
+      <c r="H62" s="32">
         <v>1.22</v>
       </c>
-      <c r="I62" s="31">
+      <c r="I62" s="32">
         <v>1.22</v>
       </c>
-      <c r="J62" s="31">
+      <c r="J62" s="32">
         <v>1.26</v>
       </c>
-      <c r="K62" s="31">
+      <c r="K62" s="32">
         <v>1.42</v>
       </c>
-      <c r="L62" s="31">
+      <c r="L62" s="32">
         <v>1.11</v>
       </c>
-      <c r="M62" s="31">
+      <c r="M62" s="32">
         <v>1.16</v>
       </c>
-      <c r="N62" s="31">
+      <c r="N62" s="32">
         <v>0.82</v>
       </c>
-      <c r="O62" s="31">
+      <c r="O62" s="32">
         <v>0.47</v>
       </c>
-      <c r="P62" s="31">
+      <c r="P62" s="32">
         <v>0.49</v>
       </c>
-      <c r="Q62" s="31">
+      <c r="Q62" s="32">
         <v>0.39</v>
       </c>
-      <c r="R62" s="31">
+      <c r="R62" s="32">
         <v>0.27</v>
       </c>
-      <c r="S62" s="31">
+      <c r="S62" s="32">
         <v>0.4</v>
       </c>
-      <c r="T62" s="31">
+      <c r="T62" s="32">
         <v>0.83</v>
       </c>
-      <c r="U62" s="29"/>
+      <c r="U62" s="30"/>
     </row>
     <row r="63" ht="15.0" customHeight="1">
-      <c r="A63" s="28" t="s">
-        <v>391</v>
-      </c>
-      <c r="B63" s="31">
+      <c r="A63" s="29" t="s">
+        <v>392</v>
+      </c>
+      <c r="B63" s="32">
         <v>1.45</v>
       </c>
-      <c r="C63" s="31">
+      <c r="C63" s="32">
         <v>1.39</v>
       </c>
-      <c r="D63" s="31">
+      <c r="D63" s="32">
         <v>1.38</v>
       </c>
-      <c r="E63" s="31">
+      <c r="E63" s="32">
         <v>1.47</v>
       </c>
-      <c r="F63" s="31">
+      <c r="F63" s="32">
         <v>1.42</v>
       </c>
-      <c r="G63" s="31">
+      <c r="G63" s="32">
         <v>1.37</v>
       </c>
-      <c r="H63" s="31">
+      <c r="H63" s="32">
         <v>1.25</v>
       </c>
-      <c r="I63" s="31">
+      <c r="I63" s="32">
         <v>1.24</v>
       </c>
-      <c r="J63" s="31">
+      <c r="J63" s="32">
         <v>1.17</v>
       </c>
-      <c r="K63" s="31">
+      <c r="K63" s="32">
         <v>1.01</v>
       </c>
-      <c r="L63" s="31">
+      <c r="L63" s="32">
         <v>0.82</v>
       </c>
-      <c r="M63" s="31">
+      <c r="M63" s="32">
         <v>0.67</v>
       </c>
-      <c r="N63" s="31">
+      <c r="N63" s="32">
         <v>0.49</v>
       </c>
-      <c r="O63" s="31">
+      <c r="O63" s="32">
         <v>0.4</v>
       </c>
-      <c r="P63" s="31">
+      <c r="P63" s="32">
         <v>0.45</v>
       </c>
-      <c r="Q63" s="29"/>
-      <c r="R63" s="29"/>
-      <c r="S63" s="29"/>
-      <c r="T63" s="29"/>
-      <c r="U63" s="29"/>
+      <c r="Q63" s="30"/>
+      <c r="R63" s="30"/>
+      <c r="S63" s="30"/>
+      <c r="T63" s="30"/>
+      <c r="U63" s="30"/>
     </row>
     <row r="64" ht="15.0" customHeight="1">
-      <c r="A64" s="26" t="s">
-        <v>392</v>
-      </c>
-      <c r="B64" s="27"/>
-      <c r="C64" s="27"/>
-      <c r="D64" s="27"/>
-      <c r="E64" s="27"/>
-      <c r="F64" s="27"/>
-      <c r="G64" s="27"/>
-      <c r="H64" s="27"/>
-      <c r="I64" s="27"/>
-      <c r="J64" s="27"/>
-      <c r="K64" s="27"/>
-      <c r="L64" s="27"/>
-      <c r="M64" s="27"/>
-      <c r="N64" s="27"/>
-      <c r="O64" s="27"/>
-      <c r="P64" s="27"/>
-      <c r="Q64" s="27"/>
-      <c r="R64" s="27"/>
-      <c r="S64" s="27"/>
-      <c r="T64" s="27"/>
-      <c r="U64" s="27"/>
+      <c r="A64" s="27" t="s">
+        <v>393</v>
+      </c>
+      <c r="B64" s="28"/>
+      <c r="C64" s="28"/>
+      <c r="D64" s="28"/>
+      <c r="E64" s="28"/>
+      <c r="F64" s="28"/>
+      <c r="G64" s="28"/>
+      <c r="H64" s="28"/>
+      <c r="I64" s="28"/>
+      <c r="J64" s="28"/>
+      <c r="K64" s="28"/>
+      <c r="L64" s="28"/>
+      <c r="M64" s="28"/>
+      <c r="N64" s="28"/>
+      <c r="O64" s="28"/>
+      <c r="P64" s="28"/>
+      <c r="Q64" s="28"/>
+      <c r="R64" s="28"/>
+      <c r="S64" s="28"/>
+      <c r="T64" s="28"/>
+      <c r="U64" s="28"/>
     </row>
     <row r="65" ht="15.0" customHeight="1">
-      <c r="A65" s="28" t="s">
-        <v>393</v>
-      </c>
-      <c r="B65" s="31">
+      <c r="A65" s="29" t="s">
+        <v>394</v>
+      </c>
+      <c r="B65" s="32">
         <v>14.53</v>
       </c>
-      <c r="C65" s="31">
+      <c r="C65" s="32">
         <v>12.3</v>
       </c>
-      <c r="D65" s="31">
+      <c r="D65" s="32">
         <v>14.09</v>
       </c>
-      <c r="E65" s="31">
+      <c r="E65" s="32">
         <v>16.14</v>
       </c>
-      <c r="F65" s="31">
+      <c r="F65" s="32">
         <v>15.62</v>
       </c>
-      <c r="G65" s="31">
+      <c r="G65" s="32">
         <v>17.29</v>
       </c>
-      <c r="H65" s="31">
+      <c r="H65" s="32">
         <v>13.44</v>
       </c>
-      <c r="I65" s="31">
+      <c r="I65" s="32">
         <v>14.18</v>
       </c>
-      <c r="J65" s="31">
+      <c r="J65" s="32">
         <v>13.32</v>
       </c>
-      <c r="K65" s="31">
+      <c r="K65" s="32">
         <v>15.9</v>
       </c>
-      <c r="L65" s="31">
+      <c r="L65" s="32">
         <v>12.86</v>
       </c>
-      <c r="M65" s="31">
+      <c r="M65" s="32">
         <v>13.1</v>
       </c>
-      <c r="N65" s="31">
+      <c r="N65" s="32">
         <v>10.46</v>
       </c>
-      <c r="O65" s="31">
+      <c r="O65" s="32">
         <v>6.27</v>
       </c>
-      <c r="P65" s="31">
+      <c r="P65" s="32">
         <v>5.74</v>
       </c>
-      <c r="Q65" s="31">
+      <c r="Q65" s="32">
         <v>3.32</v>
       </c>
-      <c r="R65" s="31">
+      <c r="R65" s="32">
         <v>8.58</v>
       </c>
-      <c r="S65" s="31">
+      <c r="S65" s="32">
         <v>4.71</v>
       </c>
-      <c r="T65" s="31">
+      <c r="T65" s="32">
         <v>13.63</v>
       </c>
-      <c r="U65" s="29"/>
+      <c r="U65" s="30"/>
     </row>
     <row r="66" ht="15.0" customHeight="1">
-      <c r="A66" s="28" t="s">
-        <v>394</v>
-      </c>
-      <c r="B66" s="31">
+      <c r="A66" s="29" t="s">
+        <v>395</v>
+      </c>
+      <c r="B66" s="32">
         <v>14.33</v>
       </c>
-      <c r="C66" s="31">
+      <c r="C66" s="32">
         <v>14.74</v>
       </c>
-      <c r="D66" s="31">
+      <c r="D66" s="32">
         <v>15.32</v>
       </c>
-      <c r="E66" s="31">
+      <c r="E66" s="32">
         <v>15.46</v>
       </c>
-      <c r="F66" s="31">
+      <c r="F66" s="32">
         <v>14.92</v>
       </c>
-      <c r="G66" s="31">
+      <c r="G66" s="32">
         <v>14.9</v>
       </c>
-      <c r="H66" s="31">
+      <c r="H66" s="32">
         <v>13.92</v>
       </c>
-      <c r="I66" s="31">
+      <c r="I66" s="32">
         <v>13.93</v>
       </c>
-      <c r="J66" s="31">
+      <c r="J66" s="32">
         <v>13.3</v>
       </c>
-      <c r="K66" s="31">
+      <c r="K66" s="32">
         <v>12.09</v>
       </c>
-      <c r="L66" s="31">
+      <c r="L66" s="32">
         <v>9.92</v>
       </c>
-      <c r="M66" s="31">
+      <c r="M66" s="32">
         <v>7.56</v>
       </c>
-      <c r="N66" s="31">
+      <c r="N66" s="32">
         <v>6.36</v>
       </c>
-      <c r="O66" s="31">
+      <c r="O66" s="32">
         <v>5.16</v>
       </c>
-      <c r="P66" s="31">
+      <c r="P66" s="32">
         <v>5.94</v>
       </c>
-      <c r="Q66" s="29"/>
-      <c r="R66" s="29"/>
-      <c r="S66" s="29"/>
-      <c r="T66" s="29"/>
-      <c r="U66" s="29"/>
+      <c r="Q66" s="30"/>
+      <c r="R66" s="30"/>
+      <c r="S66" s="30"/>
+      <c r="T66" s="30"/>
+      <c r="U66" s="30"/>
     </row>
     <row r="67" ht="15.0" customHeight="1">
-      <c r="A67" s="26" t="s">
-        <v>395</v>
-      </c>
-      <c r="B67" s="27"/>
-      <c r="C67" s="27"/>
-      <c r="D67" s="27"/>
-      <c r="E67" s="27"/>
-      <c r="F67" s="27"/>
-      <c r="G67" s="27"/>
-      <c r="H67" s="27"/>
-      <c r="I67" s="27"/>
-      <c r="J67" s="27"/>
-      <c r="K67" s="27"/>
-      <c r="L67" s="27"/>
-      <c r="M67" s="27"/>
-      <c r="N67" s="27"/>
-      <c r="O67" s="27"/>
-      <c r="P67" s="27"/>
-      <c r="Q67" s="27"/>
-      <c r="R67" s="27"/>
-      <c r="S67" s="27"/>
-      <c r="T67" s="27"/>
-      <c r="U67" s="27"/>
+      <c r="A67" s="27" t="s">
+        <v>396</v>
+      </c>
+      <c r="B67" s="28"/>
+      <c r="C67" s="28"/>
+      <c r="D67" s="28"/>
+      <c r="E67" s="28"/>
+      <c r="F67" s="28"/>
+      <c r="G67" s="28"/>
+      <c r="H67" s="28"/>
+      <c r="I67" s="28"/>
+      <c r="J67" s="28"/>
+      <c r="K67" s="28"/>
+      <c r="L67" s="28"/>
+      <c r="M67" s="28"/>
+      <c r="N67" s="28"/>
+      <c r="O67" s="28"/>
+      <c r="P67" s="28"/>
+      <c r="Q67" s="28"/>
+      <c r="R67" s="28"/>
+      <c r="S67" s="28"/>
+      <c r="T67" s="28"/>
+      <c r="U67" s="28"/>
     </row>
     <row r="68" ht="15.0" customHeight="1">
-      <c r="A68" s="28" t="s">
-        <v>396</v>
-      </c>
-      <c r="B68" s="31">
+      <c r="A68" s="29" t="s">
+        <v>397</v>
+      </c>
+      <c r="B68" s="32">
         <v>35.57</v>
       </c>
-      <c r="C68" s="31">
+      <c r="C68" s="32">
         <v>11.55</v>
       </c>
-      <c r="D68" s="29"/>
-      <c r="E68" s="30">
+      <c r="D68" s="30"/>
+      <c r="E68" s="31">
         <v>106.51</v>
       </c>
-      <c r="F68" s="31">
+      <c r="F68" s="32">
         <v>22.56</v>
       </c>
-      <c r="G68" s="31">
+      <c r="G68" s="32">
         <v>31.4</v>
       </c>
-      <c r="H68" s="31">
+      <c r="H68" s="32">
         <v>30.92</v>
       </c>
-      <c r="I68" s="31">
+      <c r="I68" s="32">
         <v>29.38</v>
       </c>
-      <c r="J68" s="31">
+      <c r="J68" s="32">
         <v>23.0</v>
       </c>
-      <c r="K68" s="31">
+      <c r="K68" s="32">
         <v>16.45</v>
       </c>
-      <c r="L68" s="31">
+      <c r="L68" s="32">
         <v>28.65</v>
       </c>
-      <c r="M68" s="31">
+      <c r="M68" s="32">
         <v>14.71</v>
       </c>
-      <c r="N68" s="31">
+      <c r="N68" s="32">
         <v>8.98</v>
       </c>
-      <c r="O68" s="29"/>
-      <c r="P68" s="31">
+      <c r="O68" s="30"/>
+      <c r="P68" s="32">
         <v>9.59</v>
       </c>
-      <c r="Q68" s="31">
+      <c r="Q68" s="32">
         <v>2.75</v>
       </c>
-      <c r="R68" s="30">
+      <c r="R68" s="31">
         <v>269.28</v>
       </c>
-      <c r="S68" s="29"/>
-      <c r="T68" s="31">
+      <c r="S68" s="30"/>
+      <c r="T68" s="32">
         <v>51.29</v>
       </c>
-      <c r="U68" s="29"/>
+      <c r="U68" s="30"/>
     </row>
     <row r="69" ht="15.0" customHeight="1">
-      <c r="A69" s="28" t="s">
-        <v>397</v>
-      </c>
-      <c r="B69" s="31">
+      <c r="A69" s="29" t="s">
+        <v>398</v>
+      </c>
+      <c r="B69" s="32">
         <v>29.31</v>
       </c>
-      <c r="C69" s="31">
+      <c r="C69" s="32">
         <v>28.08</v>
       </c>
-      <c r="D69" s="31">
+      <c r="D69" s="32">
         <v>45.89</v>
       </c>
-      <c r="E69" s="31">
+      <c r="E69" s="32">
         <v>34.19</v>
       </c>
-      <c r="F69" s="31">
+      <c r="F69" s="32">
         <v>26.99</v>
       </c>
-      <c r="G69" s="31">
+      <c r="G69" s="32">
         <v>25.59</v>
       </c>
-      <c r="H69" s="31">
+      <c r="H69" s="32">
         <v>24.4</v>
       </c>
-      <c r="I69" s="31">
+      <c r="I69" s="32">
         <v>21.14</v>
       </c>
-      <c r="J69" s="31">
+      <c r="J69" s="32">
         <v>16.85</v>
       </c>
-      <c r="K69" s="31">
+      <c r="K69" s="32">
         <v>18.05</v>
       </c>
-      <c r="L69" s="31">
+      <c r="L69" s="32">
         <v>17.14</v>
       </c>
-      <c r="M69" s="31">
+      <c r="M69" s="32">
         <v>9.82</v>
       </c>
-      <c r="N69" s="31">
+      <c r="N69" s="32">
         <v>9.36</v>
       </c>
-      <c r="O69" s="31">
+      <c r="O69" s="32">
         <v>13.35</v>
       </c>
-      <c r="P69" s="31">
+      <c r="P69" s="32">
         <v>11.4</v>
       </c>
-      <c r="Q69" s="29"/>
-      <c r="R69" s="29"/>
-      <c r="S69" s="29"/>
-      <c r="T69" s="29"/>
-      <c r="U69" s="29"/>
+      <c r="Q69" s="30"/>
+      <c r="R69" s="30"/>
+      <c r="S69" s="30"/>
+      <c r="T69" s="30"/>
+      <c r="U69" s="30"/>
     </row>
     <row r="70" ht="15.0" customHeight="1">
-      <c r="A70" s="26" t="s">
-        <v>398</v>
-      </c>
-      <c r="B70" s="27"/>
-      <c r="C70" s="27"/>
-      <c r="D70" s="27"/>
-      <c r="E70" s="27"/>
-      <c r="F70" s="27"/>
-      <c r="G70" s="27"/>
-      <c r="H70" s="27"/>
-      <c r="I70" s="27"/>
-      <c r="J70" s="27"/>
-      <c r="K70" s="27"/>
-      <c r="L70" s="27"/>
-      <c r="M70" s="27"/>
-      <c r="N70" s="27"/>
-      <c r="O70" s="27"/>
-      <c r="P70" s="27"/>
-      <c r="Q70" s="27"/>
-      <c r="R70" s="27"/>
-      <c r="S70" s="27"/>
-      <c r="T70" s="27"/>
-      <c r="U70" s="27"/>
+      <c r="A70" s="27" t="s">
+        <v>399</v>
+      </c>
+      <c r="B70" s="28"/>
+      <c r="C70" s="28"/>
+      <c r="D70" s="28"/>
+      <c r="E70" s="28"/>
+      <c r="F70" s="28"/>
+      <c r="G70" s="28"/>
+      <c r="H70" s="28"/>
+      <c r="I70" s="28"/>
+      <c r="J70" s="28"/>
+      <c r="K70" s="28"/>
+      <c r="L70" s="28"/>
+      <c r="M70" s="28"/>
+      <c r="N70" s="28"/>
+      <c r="O70" s="28"/>
+      <c r="P70" s="28"/>
+      <c r="Q70" s="28"/>
+      <c r="R70" s="28"/>
+      <c r="S70" s="28"/>
+      <c r="T70" s="28"/>
+      <c r="U70" s="28"/>
     </row>
     <row r="71" ht="15.0" customHeight="1">
-      <c r="A71" s="28" t="s">
-        <v>399</v>
-      </c>
-      <c r="B71" s="31">
+      <c r="A71" s="29" t="s">
+        <v>400</v>
+      </c>
+      <c r="B71" s="32">
         <v>75.56</v>
       </c>
-      <c r="C71" s="31">
+      <c r="C71" s="32">
         <v>15.09</v>
       </c>
-      <c r="D71" s="29"/>
-      <c r="E71" s="29"/>
-      <c r="F71" s="31">
+      <c r="D71" s="30"/>
+      <c r="E71" s="30"/>
+      <c r="F71" s="32">
         <v>35.63</v>
       </c>
-      <c r="G71" s="31">
+      <c r="G71" s="32">
         <v>64.62</v>
       </c>
-      <c r="H71" s="31">
+      <c r="H71" s="32">
         <v>92.34</v>
       </c>
-      <c r="I71" s="30">
+      <c r="I71" s="31">
         <v>114.48</v>
       </c>
-      <c r="J71" s="30">
+      <c r="J71" s="31">
         <v>118.2</v>
       </c>
-      <c r="K71" s="31">
+      <c r="K71" s="32">
         <v>38.48</v>
       </c>
-      <c r="L71" s="30">
+      <c r="L71" s="31">
         <v>213.19</v>
       </c>
-      <c r="M71" s="31">
+      <c r="M71" s="32">
         <v>25.67</v>
       </c>
-      <c r="N71" s="31">
+      <c r="N71" s="32">
         <v>11.87</v>
       </c>
-      <c r="O71" s="29"/>
-      <c r="P71" s="31">
+      <c r="O71" s="30"/>
+      <c r="P71" s="32">
         <v>17.2</v>
       </c>
-      <c r="Q71" s="31">
+      <c r="Q71" s="32">
         <v>3.2</v>
       </c>
-      <c r="R71" s="29"/>
-      <c r="S71" s="29"/>
-      <c r="T71" s="29"/>
-      <c r="U71" s="29"/>
+      <c r="R71" s="30"/>
+      <c r="S71" s="30"/>
+      <c r="T71" s="30"/>
+      <c r="U71" s="30"/>
     </row>
     <row r="72" ht="15.0" customHeight="1">
-      <c r="A72" s="28" t="s">
-        <v>400</v>
-      </c>
-      <c r="B72" s="31">
+      <c r="A72" s="29" t="s">
+        <v>401</v>
+      </c>
+      <c r="B72" s="32">
         <v>58.8</v>
       </c>
-      <c r="C72" s="31">
+      <c r="C72" s="32">
         <v>55.78</v>
       </c>
-      <c r="D72" s="30">
+      <c r="D72" s="31">
         <v>235.97</v>
       </c>
-      <c r="E72" s="31">
+      <c r="E72" s="32">
         <v>83.39</v>
       </c>
-      <c r="F72" s="31">
+      <c r="F72" s="32">
         <v>64.51</v>
       </c>
-      <c r="G72" s="31">
+      <c r="G72" s="32">
         <v>71.94</v>
       </c>
-      <c r="H72" s="31">
+      <c r="H72" s="32">
         <v>82.81</v>
       </c>
-      <c r="I72" s="31">
+      <c r="I72" s="32">
         <v>60.86</v>
       </c>
-      <c r="J72" s="31">
+      <c r="J72" s="32">
         <v>36.64</v>
       </c>
-      <c r="K72" s="31">
+      <c r="K72" s="32">
         <v>43.09</v>
       </c>
-      <c r="L72" s="31">
+      <c r="L72" s="32">
         <v>38.81</v>
       </c>
-      <c r="M72" s="31">
+      <c r="M72" s="32">
         <v>15.07</v>
       </c>
-      <c r="N72" s="31">
+      <c r="N72" s="32">
         <v>16.0</v>
       </c>
-      <c r="O72" s="31">
+      <c r="O72" s="32">
         <v>90.25</v>
       </c>
-      <c r="P72" s="31">
+      <c r="P72" s="32">
         <v>44.12</v>
       </c>
-      <c r="Q72" s="29"/>
-      <c r="R72" s="29"/>
-      <c r="S72" s="29"/>
-      <c r="T72" s="29"/>
-      <c r="U72" s="29"/>
+      <c r="Q72" s="30"/>
+      <c r="R72" s="30"/>
+      <c r="S72" s="30"/>
+      <c r="T72" s="30"/>
+      <c r="U72" s="30"/>
     </row>
     <row r="73" ht="15.75" customHeight="1"/>
     <row r="74" ht="15.75" customHeight="1"/>

</xml_diff>